<commit_message>
feat: actualizar templates Excel Humedad, EquiArena y Proctor con retoques visuales
</commit_message>
<xml_diff>
--- a/app/templates/informes/EquiArena/1-INF.-N-000-26-SU21-E.-ARENA-V08.xlsx
+++ b/app/templates/informes/EquiArena/1-INF.-N-000-26-SU21-E.-ARENA-V08.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\3.0 Formatos e informes\2026\1.0 Informe de ensayo\1.1 Informe Suelo\INFORME ACREDITADO-E ISO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\informes\EquiArena\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C4813B6-51FD-4DEF-91D9-7E6E91CFE9AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B33F4E50-C0BB-4C21-BAEE-5C0C7EE2931B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="556" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="556" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FORMATO" sheetId="97" r:id="rId1"/>
@@ -2945,6 +2945,115 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="44" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="44" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="44" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="1"/>
@@ -2981,114 +3090,72 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="19" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="19" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="19" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="44" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="44" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="44" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3131,73 +3198,6 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="19" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="19" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="19" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4648,7 +4648,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -4707,7 +4707,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="datos de ecuacion del anillo"/>
@@ -4826,7 +4826,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -4877,7 +4877,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -4929,7 +4929,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink5.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="BGA"/>
@@ -4961,7 +4961,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink6.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -5666,23 +5666,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0883903-CEA4-449A-A5F8-47E41E2F4676}">
   <dimension ref="A1:N56"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.28515625" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.33203125" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.85546875" style="199" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" style="199" customWidth="1"/>
-    <col min="3" max="3" width="5.7109375" style="199" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" style="199" customWidth="1"/>
-    <col min="5" max="5" width="8.140625" style="199" customWidth="1"/>
-    <col min="6" max="6" width="11.28515625" style="199" customWidth="1"/>
-    <col min="7" max="7" width="11.140625" style="199" customWidth="1"/>
+    <col min="1" max="1" width="6.88671875" style="199" customWidth="1"/>
+    <col min="2" max="2" width="9.109375" style="199" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" style="199" customWidth="1"/>
+    <col min="4" max="4" width="10.109375" style="199" customWidth="1"/>
+    <col min="5" max="5" width="8.109375" style="199" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" style="199" customWidth="1"/>
+    <col min="7" max="7" width="11.109375" style="199" customWidth="1"/>
     <col min="8" max="10" width="13" style="199" customWidth="1"/>
-    <col min="11" max="11" width="6.42578125" style="199" customWidth="1"/>
-    <col min="12" max="12" width="9.42578125" style="199" customWidth="1"/>
-    <col min="13" max="14" width="10.7109375" style="199" customWidth="1"/>
-    <col min="15" max="16384" width="10.28515625" style="199"/>
+    <col min="11" max="11" width="6.44140625" style="199" customWidth="1"/>
+    <col min="12" max="12" width="9.44140625" style="199" customWidth="1"/>
+    <col min="13" max="14" width="10.6640625" style="199" customWidth="1"/>
+    <col min="15" max="16384" width="10.33203125" style="199"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A1" s="195"/>
       <c r="B1" s="196"/>
       <c r="C1" s="196"/>
@@ -5694,7 +5694,7 @@
       <c r="I1" s="197"/>
       <c r="J1" s="198"/>
     </row>
-    <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="200"/>
       <c r="B2" s="201"/>
       <c r="C2" s="201"/>
@@ -5710,7 +5710,7 @@
       </c>
       <c r="N2" s="280"/>
     </row>
-    <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="200"/>
       <c r="B3" s="201"/>
       <c r="C3" s="201"/>
@@ -5726,7 +5726,7 @@
       </c>
       <c r="N3" s="281"/>
     </row>
-    <row r="4" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="200"/>
       <c r="B4" s="201"/>
       <c r="C4" s="201"/>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="N4" s="281"/>
     </row>
-    <row r="5" spans="1:14" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="204"/>
       <c r="B5" s="205"/>
       <c r="C5" s="205"/>
@@ -5758,7 +5758,7 @@
       </c>
       <c r="N5" s="281"/>
     </row>
-    <row r="6" spans="1:14" ht="5.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" ht="5.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A6" s="207"/>
       <c r="B6" s="207"/>
       <c r="C6" s="207"/>
@@ -5772,43 +5772,43 @@
       <c r="M6" s="282"/>
       <c r="N6" s="283"/>
     </row>
-    <row r="7" spans="1:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="409" t="s">
+    <row r="7" spans="1:14" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="437" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="409"/>
-      <c r="C7" s="409"/>
-      <c r="D7" s="409"/>
-      <c r="E7" s="409"/>
-      <c r="F7" s="409"/>
-      <c r="G7" s="409"/>
-      <c r="H7" s="409"/>
-      <c r="I7" s="409"/>
-      <c r="J7" s="409"/>
+      <c r="B7" s="437"/>
+      <c r="C7" s="437"/>
+      <c r="D7" s="437"/>
+      <c r="E7" s="437"/>
+      <c r="F7" s="437"/>
+      <c r="G7" s="437"/>
+      <c r="H7" s="437"/>
+      <c r="I7" s="437"/>
+      <c r="J7" s="437"/>
       <c r="M7" s="279" t="s">
         <v>119</v>
       </c>
       <c r="N7" s="283"/>
     </row>
-    <row r="8" spans="1:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="410" t="s">
+    <row r="8" spans="1:14" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="438" t="s">
         <v>122</v>
       </c>
-      <c r="B8" s="410"/>
-      <c r="C8" s="410"/>
-      <c r="D8" s="410"/>
-      <c r="E8" s="410"/>
-      <c r="F8" s="410"/>
-      <c r="G8" s="410"/>
-      <c r="H8" s="410"/>
-      <c r="I8" s="410"/>
-      <c r="J8" s="410"/>
+      <c r="B8" s="438"/>
+      <c r="C8" s="438"/>
+      <c r="D8" s="438"/>
+      <c r="E8" s="438"/>
+      <c r="F8" s="438"/>
+      <c r="G8" s="438"/>
+      <c r="H8" s="438"/>
+      <c r="I8" s="438"/>
+      <c r="J8" s="438"/>
       <c r="M8" s="279" t="s">
         <v>157</v>
       </c>
       <c r="N8" s="284"/>
     </row>
-    <row r="9" spans="1:14" ht="6.6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" ht="6.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="208"/>
       <c r="B9" s="208"/>
       <c r="C9" s="208"/>
@@ -5824,39 +5824,39 @@
       </c>
       <c r="N9" s="283"/>
     </row>
-    <row r="10" spans="1:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="411" t="s">
+    <row r="10" spans="1:14" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="439" t="s">
         <v>123</v>
       </c>
-      <c r="C10" s="411"/>
-      <c r="D10" s="411" t="s">
+      <c r="C10" s="439"/>
+      <c r="D10" s="439" t="s">
         <v>124</v>
       </c>
-      <c r="E10" s="411"/>
-      <c r="F10" s="411" t="s">
+      <c r="E10" s="439"/>
+      <c r="F10" s="439" t="s">
         <v>125</v>
       </c>
-      <c r="G10" s="411"/>
-      <c r="H10" s="411" t="s">
+      <c r="G10" s="439"/>
+      <c r="H10" s="439" t="s">
         <v>126</v>
       </c>
-      <c r="I10" s="411"/>
+      <c r="I10" s="439"/>
       <c r="J10" s="209"/>
       <c r="K10" s="210"/>
       <c r="L10" s="210"/>
       <c r="M10" s="282"/>
       <c r="N10" s="283"/>
     </row>
-    <row r="11" spans="1:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="211"/>
-      <c r="B11" s="411"/>
-      <c r="C11" s="411"/>
-      <c r="D11" s="411"/>
-      <c r="E11" s="411"/>
-      <c r="F11" s="411"/>
-      <c r="G11" s="411"/>
-      <c r="H11" s="411"/>
-      <c r="I11" s="411"/>
+      <c r="B11" s="439"/>
+      <c r="C11" s="439"/>
+      <c r="D11" s="439"/>
+      <c r="E11" s="439"/>
+      <c r="F11" s="439"/>
+      <c r="G11" s="439"/>
+      <c r="H11" s="439"/>
+      <c r="I11" s="439"/>
       <c r="J11" s="212"/>
       <c r="K11" s="210"/>
       <c r="L11" s="210"/>
@@ -5865,7 +5865,7 @@
       </c>
       <c r="N11" s="283"/>
     </row>
-    <row r="12" spans="1:14" ht="7.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" ht="7.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="211"/>
       <c r="B12" s="211"/>
       <c r="C12" s="213"/>
@@ -5883,19 +5883,19 @@
       </c>
       <c r="N12" s="284"/>
     </row>
-    <row r="13" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="412" t="s">
+    <row r="13" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="440" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="413"/>
-      <c r="C13" s="413"/>
-      <c r="D13" s="413"/>
-      <c r="E13" s="413"/>
-      <c r="F13" s="413"/>
-      <c r="G13" s="413"/>
-      <c r="H13" s="413"/>
-      <c r="I13" s="413"/>
-      <c r="J13" s="414"/>
+      <c r="B13" s="441"/>
+      <c r="C13" s="441"/>
+      <c r="D13" s="441"/>
+      <c r="E13" s="441"/>
+      <c r="F13" s="441"/>
+      <c r="G13" s="441"/>
+      <c r="H13" s="441"/>
+      <c r="I13" s="441"/>
+      <c r="J13" s="442"/>
       <c r="K13" s="210"/>
       <c r="L13" s="210"/>
       <c r="M13" s="279" t="s">
@@ -5903,25 +5903,25 @@
       </c>
       <c r="N13" s="284"/>
     </row>
-    <row r="14" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="406" t="s">
+    <row r="14" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="434" t="s">
         <v>117</v>
       </c>
-      <c r="B14" s="407"/>
-      <c r="C14" s="407"/>
-      <c r="D14" s="407"/>
-      <c r="E14" s="407"/>
-      <c r="F14" s="407"/>
-      <c r="G14" s="407"/>
-      <c r="H14" s="407"/>
-      <c r="I14" s="407"/>
-      <c r="J14" s="408"/>
+      <c r="B14" s="435"/>
+      <c r="C14" s="435"/>
+      <c r="D14" s="435"/>
+      <c r="E14" s="435"/>
+      <c r="F14" s="435"/>
+      <c r="G14" s="435"/>
+      <c r="H14" s="435"/>
+      <c r="I14" s="435"/>
+      <c r="J14" s="436"/>
       <c r="K14" s="210"/>
       <c r="L14" s="210"/>
       <c r="M14" s="282"/>
       <c r="N14" s="283"/>
     </row>
-    <row r="15" spans="1:14" ht="6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" ht="6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="216"/>
       <c r="B15" s="217"/>
       <c r="C15" s="218"/>
@@ -5939,23 +5939,23 @@
       </c>
       <c r="N15" s="285"/>
     </row>
-    <row r="16" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="221"/>
-      <c r="B16" s="415" t="s">
+      <c r="B16" s="426" t="s">
         <v>118</v>
       </c>
-      <c r="C16" s="415"/>
-      <c r="D16" s="415"/>
+      <c r="C16" s="426"/>
+      <c r="D16" s="426"/>
       <c r="E16" s="222"/>
-      <c r="F16" s="416" t="s">
+      <c r="F16" s="427" t="s">
         <v>127</v>
       </c>
-      <c r="G16" s="416"/>
+      <c r="G16" s="427"/>
       <c r="H16" s="222"/>
-      <c r="I16" s="417" t="s">
+      <c r="I16" s="428" t="s">
         <v>128</v>
       </c>
-      <c r="J16" s="420"/>
+      <c r="J16" s="431"/>
       <c r="K16" s="210"/>
       <c r="L16" s="210"/>
       <c r="M16" s="279" t="s">
@@ -5963,17 +5963,17 @@
       </c>
       <c r="N16" s="285"/>
     </row>
-    <row r="17" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="221"/>
-      <c r="B17" s="423"/>
-      <c r="C17" s="424"/>
-      <c r="D17" s="425"/>
+      <c r="B17" s="417"/>
+      <c r="C17" s="418"/>
+      <c r="D17" s="419"/>
       <c r="E17" s="223"/>
-      <c r="F17" s="423"/>
-      <c r="G17" s="425"/>
+      <c r="F17" s="417"/>
+      <c r="G17" s="419"/>
       <c r="H17" s="222"/>
-      <c r="I17" s="418"/>
-      <c r="J17" s="421"/>
+      <c r="I17" s="429"/>
+      <c r="J17" s="432"/>
       <c r="K17" s="210"/>
       <c r="L17" s="210"/>
       <c r="M17" s="279" t="s">
@@ -5981,17 +5981,17 @@
       </c>
       <c r="N17" s="286"/>
     </row>
-    <row r="18" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E18" s="223"/>
       <c r="F18" s="223"/>
       <c r="G18" s="223"/>
       <c r="H18" s="222"/>
-      <c r="I18" s="419"/>
-      <c r="J18" s="422"/>
+      <c r="I18" s="430"/>
+      <c r="J18" s="433"/>
       <c r="L18" s="210"/>
       <c r="M18" s="224"/>
     </row>
-    <row r="19" spans="1:14" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:14" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="225"/>
       <c r="B19" s="223"/>
       <c r="C19" s="223"/>
@@ -6005,13 +6005,13 @@
       <c r="L19" s="210"/>
       <c r="M19" s="224"/>
     </row>
-    <row r="20" spans="1:14" s="228" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:14" s="228" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="227"/>
-      <c r="B20" s="426" t="s">
+      <c r="B20" s="413" t="s">
         <v>129</v>
       </c>
-      <c r="C20" s="426"/>
-      <c r="D20" s="428"/>
+      <c r="C20" s="413"/>
+      <c r="D20" s="415"/>
       <c r="F20" s="229" t="s">
         <v>130</v>
       </c>
@@ -6022,20 +6022,20 @@
       <c r="L20" s="231"/>
       <c r="M20" s="224"/>
     </row>
-    <row r="21" spans="1:14" s="228" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:14" s="228" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="232"/>
-      <c r="B21" s="427"/>
-      <c r="C21" s="427"/>
-      <c r="D21" s="429"/>
-      <c r="F21" s="423"/>
-      <c r="G21" s="424"/>
-      <c r="H21" s="425"/>
+      <c r="B21" s="414"/>
+      <c r="C21" s="414"/>
+      <c r="D21" s="416"/>
+      <c r="F21" s="417"/>
+      <c r="G21" s="418"/>
+      <c r="H21" s="419"/>
       <c r="I21" s="230"/>
       <c r="J21" s="226"/>
       <c r="L21" s="231"/>
       <c r="M21" s="224"/>
     </row>
-    <row r="22" spans="1:14" s="228" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:14" s="228" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="232"/>
       <c r="B22" s="230"/>
       <c r="C22" s="230"/>
@@ -6045,7 +6045,7 @@
       <c r="L22" s="231"/>
       <c r="M22" s="224"/>
     </row>
-    <row r="23" spans="1:14" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:14" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="233"/>
       <c r="B23" s="234"/>
       <c r="C23" s="234"/>
@@ -6058,14 +6058,14 @@
       <c r="J23" s="235"/>
       <c r="L23" s="236"/>
     </row>
-    <row r="24" spans="1:14" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:14" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="67"/>
       <c r="B24" s="67"/>
       <c r="J24" s="67"/>
       <c r="K24" s="210"/>
       <c r="L24" s="237"/>
     </row>
-    <row r="25" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="238" t="s">
         <v>131</v>
       </c>
@@ -6089,7 +6089,7 @@
       <c r="K25" s="244"/>
       <c r="L25" s="245"/>
     </row>
-    <row r="26" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="246" t="s">
         <v>135</v>
       </c>
@@ -6109,7 +6109,7 @@
       <c r="K26" s="252"/>
       <c r="N26" s="253"/>
     </row>
-    <row r="27" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="246" t="s">
         <v>136</v>
       </c>
@@ -6129,7 +6129,7 @@
       <c r="K27" s="255"/>
       <c r="L27" s="253"/>
     </row>
-    <row r="28" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="246" t="s">
         <v>138</v>
       </c>
@@ -6149,7 +6149,7 @@
       <c r="K28" s="257"/>
       <c r="L28" s="253"/>
     </row>
-    <row r="29" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="246" t="s">
         <v>139</v>
       </c>
@@ -6169,7 +6169,7 @@
       <c r="K29" s="257"/>
       <c r="L29" s="236"/>
     </row>
-    <row r="30" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="246" t="s">
         <v>14</v>
       </c>
@@ -6189,7 +6189,7 @@
       <c r="K30" s="257"/>
       <c r="L30" s="210"/>
     </row>
-    <row r="31" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="246" t="s">
         <v>15</v>
       </c>
@@ -6209,7 +6209,7 @@
       <c r="K31" s="257"/>
       <c r="L31" s="210"/>
     </row>
-    <row r="32" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="246" t="s">
         <v>140</v>
       </c>
@@ -6229,7 +6229,7 @@
       <c r="K32" s="258"/>
       <c r="L32" s="210"/>
     </row>
-    <row r="33" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="246" t="s">
         <v>141</v>
       </c>
@@ -6249,7 +6249,7 @@
       <c r="K33" s="262"/>
       <c r="L33" s="210"/>
     </row>
-    <row r="34" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="246" t="s">
         <v>142</v>
       </c>
@@ -6269,7 +6269,7 @@
       <c r="K34" s="264"/>
       <c r="L34" s="210"/>
     </row>
-    <row r="35" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="246" t="s">
         <v>143</v>
       </c>
@@ -6289,7 +6289,7 @@
       <c r="K35" s="210"/>
       <c r="L35" s="210"/>
     </row>
-    <row r="36" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="246" t="s">
         <v>145</v>
       </c>
@@ -6303,15 +6303,15 @@
       <c r="G36" s="250" t="s">
         <v>1</v>
       </c>
-      <c r="H36" s="430">
+      <c r="H36" s="420">
         <v>31</v>
       </c>
-      <c r="I36" s="431"/>
-      <c r="J36" s="432"/>
+      <c r="I36" s="421"/>
+      <c r="J36" s="422"/>
       <c r="K36" s="210"/>
       <c r="L36" s="210"/>
     </row>
-    <row r="37" spans="1:12" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:12" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="267"/>
       <c r="B37" s="267"/>
       <c r="C37" s="268"/>
@@ -6325,16 +6325,16 @@
       <c r="K37" s="210"/>
       <c r="L37" s="210"/>
     </row>
-    <row r="38" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="433" t="s">
+    <row r="38" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="423" t="s">
         <v>146</v>
       </c>
-      <c r="B38" s="434"/>
-      <c r="C38" s="435"/>
-      <c r="D38" s="433" t="s">
+      <c r="B38" s="424"/>
+      <c r="C38" s="425"/>
+      <c r="D38" s="423" t="s">
         <v>147</v>
       </c>
-      <c r="E38" s="435"/>
+      <c r="E38" s="425"/>
       <c r="F38" s="271" t="s">
         <v>100</v>
       </c>
@@ -6345,14 +6345,14 @@
       <c r="K38" s="210"/>
       <c r="L38" s="210"/>
     </row>
-    <row r="39" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="436" t="s">
+    <row r="39" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="406" t="s">
         <v>148</v>
       </c>
-      <c r="B39" s="437"/>
-      <c r="C39" s="438"/>
-      <c r="D39" s="436"/>
-      <c r="E39" s="438"/>
+      <c r="B39" s="407"/>
+      <c r="C39" s="408"/>
+      <c r="D39" s="406"/>
+      <c r="E39" s="408"/>
       <c r="F39" s="233"/>
       <c r="G39" s="234"/>
       <c r="H39" s="234"/>
@@ -6361,14 +6361,14 @@
       <c r="K39" s="210"/>
       <c r="L39" s="210"/>
     </row>
-    <row r="40" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="436" t="s">
+    <row r="40" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="406" t="s">
         <v>149</v>
       </c>
-      <c r="B40" s="437"/>
-      <c r="C40" s="438"/>
-      <c r="D40" s="436"/>
-      <c r="E40" s="438"/>
+      <c r="B40" s="407"/>
+      <c r="C40" s="408"/>
+      <c r="D40" s="406"/>
+      <c r="E40" s="408"/>
       <c r="F40" s="274"/>
       <c r="G40" s="272"/>
       <c r="H40" s="272"/>
@@ -6377,67 +6377,67 @@
       <c r="K40" s="210"/>
       <c r="L40" s="210"/>
     </row>
-    <row r="41" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="436" t="s">
+    <row r="41" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="406" t="s">
         <v>150</v>
       </c>
-      <c r="B41" s="437"/>
-      <c r="C41" s="438"/>
-      <c r="D41" s="436"/>
-      <c r="E41" s="438"/>
+      <c r="B41" s="407"/>
+      <c r="C41" s="408"/>
+      <c r="D41" s="406"/>
+      <c r="E41" s="408"/>
       <c r="F41" s="221"/>
       <c r="K41" s="210"/>
       <c r="L41" s="210"/>
     </row>
-    <row r="42" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="440" t="s">
+    <row r="42" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="410" t="s">
         <v>151</v>
       </c>
-      <c r="B42" s="441"/>
-      <c r="C42" s="442"/>
-      <c r="D42" s="436"/>
-      <c r="E42" s="438"/>
+      <c r="B42" s="411"/>
+      <c r="C42" s="412"/>
+      <c r="D42" s="406"/>
+      <c r="E42" s="408"/>
       <c r="F42" s="221"/>
       <c r="K42" s="210"/>
       <c r="L42" s="210"/>
     </row>
-    <row r="43" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="440" t="s">
+    <row r="43" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="410" t="s">
         <v>152</v>
       </c>
-      <c r="B43" s="441"/>
-      <c r="C43" s="442"/>
-      <c r="D43" s="436"/>
-      <c r="E43" s="438"/>
+      <c r="B43" s="411"/>
+      <c r="C43" s="412"/>
+      <c r="D43" s="406"/>
+      <c r="E43" s="408"/>
       <c r="F43" s="221"/>
       <c r="K43" s="210"/>
       <c r="L43" s="210"/>
     </row>
-    <row r="44" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="436" t="s">
+    <row r="44" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="406" t="s">
         <v>153</v>
       </c>
-      <c r="B44" s="437"/>
-      <c r="C44" s="438"/>
-      <c r="D44" s="436"/>
-      <c r="E44" s="438"/>
+      <c r="B44" s="407"/>
+      <c r="C44" s="408"/>
+      <c r="D44" s="406"/>
+      <c r="E44" s="408"/>
       <c r="F44" s="221"/>
       <c r="K44" s="210"/>
       <c r="L44" s="210"/>
     </row>
-    <row r="45" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="436" t="s">
+    <row r="45" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="406" t="s">
         <v>154</v>
       </c>
-      <c r="B45" s="437"/>
-      <c r="C45" s="438"/>
-      <c r="D45" s="436"/>
-      <c r="E45" s="438"/>
+      <c r="B45" s="407"/>
+      <c r="C45" s="408"/>
+      <c r="D45" s="406"/>
+      <c r="E45" s="408"/>
       <c r="F45" s="221"/>
       <c r="K45" s="210"/>
       <c r="L45" s="210"/>
     </row>
-    <row r="46" spans="1:12" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:12" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="275"/>
       <c r="B46" s="275"/>
       <c r="C46" s="270"/>
@@ -6451,7 +6451,7 @@
       <c r="K46" s="210"/>
       <c r="L46" s="210"/>
     </row>
-    <row r="47" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="276"/>
       <c r="B47" s="276"/>
       <c r="C47" s="270"/>
@@ -6459,7 +6459,7 @@
       <c r="K47" s="210"/>
       <c r="L47" s="210"/>
     </row>
-    <row r="48" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="276"/>
       <c r="B48" s="276"/>
       <c r="C48" s="270"/>
@@ -6467,7 +6467,7 @@
       <c r="K48" s="210"/>
       <c r="L48" s="210"/>
     </row>
-    <row r="49" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="276"/>
       <c r="B49" s="276"/>
       <c r="C49" s="270"/>
@@ -6475,7 +6475,7 @@
       <c r="K49" s="210"/>
       <c r="L49" s="210"/>
     </row>
-    <row r="50" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="277"/>
       <c r="B50" s="277"/>
       <c r="C50" s="270"/>
@@ -6489,7 +6489,7 @@
       <c r="K50" s="210"/>
       <c r="L50" s="210"/>
     </row>
-    <row r="51" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="278" t="s">
         <v>18</v>
       </c>
@@ -6505,7 +6505,7 @@
       <c r="K51" s="210"/>
       <c r="L51" s="210"/>
     </row>
-    <row r="52" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:12" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="278" t="s">
         <v>155</v>
       </c>
@@ -6523,23 +6523,23 @@
       <c r="K52" s="210"/>
       <c r="L52" s="210"/>
     </row>
-    <row r="53" spans="1:12" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="54" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="439" t="s">
+    <row r="53" spans="1:12" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="54" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="409" t="s">
         <v>170</v>
       </c>
-      <c r="B54" s="439"/>
-      <c r="C54" s="439"/>
-      <c r="D54" s="439"/>
-      <c r="E54" s="439"/>
-      <c r="F54" s="439"/>
-      <c r="G54" s="439"/>
-      <c r="H54" s="439"/>
-      <c r="I54" s="439"/>
-      <c r="J54" s="439"/>
-    </row>
-    <row r="55" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="56" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.2"/>
+      <c r="B54" s="409"/>
+      <c r="C54" s="409"/>
+      <c r="D54" s="409"/>
+      <c r="E54" s="409"/>
+      <c r="F54" s="409"/>
+      <c r="G54" s="409"/>
+      <c r="H54" s="409"/>
+      <c r="I54" s="409"/>
+      <c r="J54" s="409"/>
+    </row>
+    <row r="55" spans="1:12" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="1:12" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="M2qAW+U6hDKcwcOWYiT+b9VHOy6irX93erXkEpP6UPGziP4Tt89tbslkmG90DAQ/RAQXiyxyY4VI391swfT4sQ==" saltValue="qMgqI4U5/0thO9gXTFLcNw==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0"/>
   <protectedRanges>
@@ -6548,33 +6548,6 @@
     <protectedRange sqref="H31:J31" name="Rango8_1"/>
   </protectedRanges>
   <mergeCells count="39">
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="A54:J54"/>
-    <mergeCell ref="A42:C42"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="A43:C43"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="B20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="F21:H21"/>
-    <mergeCell ref="H36:J36"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="I16:I18"/>
-    <mergeCell ref="J16:J18"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="F17:G17"/>
     <mergeCell ref="A14:J14"/>
     <mergeCell ref="A7:J7"/>
     <mergeCell ref="A8:J8"/>
@@ -6587,6 +6560,33 @@
     <mergeCell ref="F11:G11"/>
     <mergeCell ref="H11:I11"/>
     <mergeCell ref="A13:J13"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="I16:I18"/>
+    <mergeCell ref="J16:J18"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="B20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="F21:H21"/>
+    <mergeCell ref="H36:J36"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="A54:J54"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="D44:E44"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0.39370078740157483" top="0" bottom="0" header="0" footer="0"/>
@@ -6601,24 +6601,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
   <dimension ref="A1:Q51"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.33203125" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.28515625" style="296" customWidth="1"/>
-    <col min="2" max="2" width="2.140625" style="296" customWidth="1"/>
-    <col min="3" max="3" width="4.5703125" style="296" customWidth="1"/>
-    <col min="4" max="4" width="1.7109375" style="296" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" style="296" customWidth="1"/>
-    <col min="6" max="6" width="10.42578125" style="296" customWidth="1"/>
-    <col min="7" max="7" width="8.140625" style="296" customWidth="1"/>
-    <col min="8" max="8" width="6.5703125" style="296" customWidth="1"/>
-    <col min="9" max="11" width="10.5703125" style="296" customWidth="1"/>
-    <col min="12" max="12" width="1.5703125" style="296" customWidth="1"/>
-    <col min="13" max="13" width="13.5703125" style="296" customWidth="1"/>
-    <col min="14" max="14" width="6.42578125" style="296" customWidth="1"/>
-    <col min="15" max="15" width="8.5703125" style="296" customWidth="1"/>
+    <col min="1" max="1" width="11.33203125" style="296" customWidth="1"/>
+    <col min="2" max="2" width="2.109375" style="296" customWidth="1"/>
+    <col min="3" max="3" width="4.5546875" style="296" customWidth="1"/>
+    <col min="4" max="4" width="1.6640625" style="296" customWidth="1"/>
+    <col min="5" max="5" width="13.88671875" style="296" customWidth="1"/>
+    <col min="6" max="6" width="10.44140625" style="296" customWidth="1"/>
+    <col min="7" max="7" width="8.109375" style="296" customWidth="1"/>
+    <col min="8" max="8" width="6.5546875" style="296" customWidth="1"/>
+    <col min="9" max="11" width="10.5546875" style="296" customWidth="1"/>
+    <col min="12" max="12" width="1.5546875" style="296" customWidth="1"/>
+    <col min="13" max="13" width="13.5546875" style="296" customWidth="1"/>
+    <col min="14" max="14" width="6.44140625" style="296" customWidth="1"/>
+    <col min="15" max="15" width="8.5546875" style="296" customWidth="1"/>
     <col min="16" max="16" width="8" style="296" customWidth="1"/>
-    <col min="17" max="17" width="13.28515625" style="296" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="10.28515625" style="296"/>
+    <col min="17" max="17" width="13.33203125" style="296" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="10.33203125" style="296"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -6637,38 +6637,38 @@
       <c r="M1" s="295"/>
     </row>
     <row r="2" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="443" t="s">
+      <c r="A2" s="464" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="443"/>
-      <c r="C2" s="443"/>
-      <c r="D2" s="443"/>
-      <c r="E2" s="443"/>
-      <c r="F2" s="443"/>
-      <c r="G2" s="443"/>
-      <c r="H2" s="443"/>
-      <c r="I2" s="443"/>
-      <c r="J2" s="443"/>
-      <c r="K2" s="443"/>
-      <c r="L2" s="443"/>
-      <c r="M2" s="443"/>
+      <c r="B2" s="464"/>
+      <c r="C2" s="464"/>
+      <c r="D2" s="464"/>
+      <c r="E2" s="464"/>
+      <c r="F2" s="464"/>
+      <c r="G2" s="464"/>
+      <c r="H2" s="464"/>
+      <c r="I2" s="464"/>
+      <c r="J2" s="464"/>
+      <c r="K2" s="464"/>
+      <c r="L2" s="464"/>
+      <c r="M2" s="464"/>
     </row>
     <row r="3" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="444">
+      <c r="A3" s="465">
         <v>0</v>
       </c>
-      <c r="B3" s="444"/>
-      <c r="C3" s="444"/>
-      <c r="D3" s="444"/>
-      <c r="E3" s="444"/>
-      <c r="F3" s="444"/>
-      <c r="G3" s="444"/>
-      <c r="H3" s="444"/>
-      <c r="I3" s="444"/>
-      <c r="J3" s="444"/>
-      <c r="K3" s="444"/>
-      <c r="L3" s="444"/>
-      <c r="M3" s="444"/>
+      <c r="B3" s="465"/>
+      <c r="C3" s="465"/>
+      <c r="D3" s="465"/>
+      <c r="E3" s="465"/>
+      <c r="F3" s="465"/>
+      <c r="G3" s="465"/>
+      <c r="H3" s="465"/>
+      <c r="I3" s="465"/>
+      <c r="J3" s="465"/>
+      <c r="K3" s="465"/>
+      <c r="L3" s="465"/>
+      <c r="M3" s="465"/>
     </row>
     <row r="4" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6678,17 +6678,17 @@
       <c r="B5" s="298" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="455">
+      <c r="C5" s="476">
         <f>+FORMATO!N2</f>
         <v>0</v>
       </c>
-      <c r="D5" s="455"/>
-      <c r="E5" s="455"/>
-      <c r="F5" s="455"/>
-      <c r="G5" s="455"/>
-      <c r="H5" s="455"/>
-      <c r="I5" s="455"/>
-      <c r="J5" s="455"/>
+      <c r="D5" s="476"/>
+      <c r="E5" s="476"/>
+      <c r="F5" s="476"/>
+      <c r="G5" s="476"/>
+      <c r="H5" s="476"/>
+      <c r="I5" s="476"/>
+      <c r="J5" s="476"/>
       <c r="K5" s="299" t="s">
         <v>20</v>
       </c>
@@ -6706,17 +6706,17 @@
       <c r="B6" s="298" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="455">
+      <c r="C6" s="476">
         <f>+FORMATO!N3</f>
         <v>0</v>
       </c>
-      <c r="D6" s="455"/>
-      <c r="E6" s="455"/>
-      <c r="F6" s="455"/>
-      <c r="G6" s="455"/>
-      <c r="H6" s="455"/>
-      <c r="I6" s="455"/>
-      <c r="J6" s="455"/>
+      <c r="D6" s="476"/>
+      <c r="E6" s="476"/>
+      <c r="F6" s="476"/>
+      <c r="G6" s="476"/>
+      <c r="H6" s="476"/>
+      <c r="I6" s="476"/>
+      <c r="J6" s="476"/>
       <c r="K6" s="279" t="s">
         <v>119</v>
       </c>
@@ -6731,24 +6731,24 @@
       <c r="O6" s="303"/>
       <c r="P6" s="303"/>
     </row>
-    <row r="7" spans="1:16" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="297" t="s">
         <v>22</v>
       </c>
       <c r="B7" s="298" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="455">
+      <c r="C7" s="476">
         <f>+FORMATO!N4</f>
         <v>0</v>
       </c>
-      <c r="D7" s="455"/>
-      <c r="E7" s="455"/>
-      <c r="F7" s="455"/>
-      <c r="G7" s="455"/>
-      <c r="H7" s="455"/>
-      <c r="I7" s="455"/>
-      <c r="J7" s="455"/>
+      <c r="D7" s="476"/>
+      <c r="E7" s="476"/>
+      <c r="F7" s="476"/>
+      <c r="G7" s="476"/>
+      <c r="H7" s="476"/>
+      <c r="I7" s="476"/>
+      <c r="J7" s="476"/>
       <c r="K7" s="279" t="s">
         <v>158</v>
       </c>
@@ -6763,24 +6763,24 @@
       <c r="O7" s="303"/>
       <c r="P7" s="303"/>
     </row>
-    <row r="8" spans="1:16" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" ht="19.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="297" t="s">
         <v>23</v>
       </c>
       <c r="B8" s="298" t="s">
         <v>0</v>
       </c>
-      <c r="C8" s="455">
+      <c r="C8" s="476">
         <f>+FORMATO!N5</f>
         <v>0</v>
       </c>
-      <c r="D8" s="455"/>
-      <c r="E8" s="455"/>
-      <c r="F8" s="455"/>
-      <c r="G8" s="455"/>
-      <c r="H8" s="455"/>
-      <c r="I8" s="455"/>
-      <c r="J8" s="455"/>
+      <c r="D8" s="476"/>
+      <c r="E8" s="476"/>
+      <c r="F8" s="476"/>
+      <c r="G8" s="476"/>
+      <c r="H8" s="476"/>
+      <c r="I8" s="476"/>
+      <c r="J8" s="476"/>
       <c r="K8" s="304" t="s">
         <v>36</v>
       </c>
@@ -6788,7 +6788,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="305">
-        <f>+FORMATO!N9</f>
+        <f>+FORMATO!N8</f>
         <v>0</v>
       </c>
       <c r="N8" s="303"/>
@@ -6816,41 +6816,41 @@
       <c r="P9" s="303"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="447" t="s">
+      <c r="A10" s="468" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="448"/>
-      <c r="C10" s="448"/>
-      <c r="D10" s="448"/>
-      <c r="E10" s="448"/>
-      <c r="F10" s="448"/>
-      <c r="G10" s="448"/>
-      <c r="H10" s="448"/>
-      <c r="I10" s="448"/>
-      <c r="J10" s="448"/>
-      <c r="K10" s="448"/>
-      <c r="L10" s="448"/>
-      <c r="M10" s="449"/>
+      <c r="B10" s="469"/>
+      <c r="C10" s="469"/>
+      <c r="D10" s="469"/>
+      <c r="E10" s="469"/>
+      <c r="F10" s="469"/>
+      <c r="G10" s="469"/>
+      <c r="H10" s="469"/>
+      <c r="I10" s="469"/>
+      <c r="J10" s="469"/>
+      <c r="K10" s="469"/>
+      <c r="L10" s="469"/>
+      <c r="M10" s="470"/>
       <c r="N10" s="303"/>
       <c r="O10" s="303"/>
       <c r="P10" s="303"/>
     </row>
     <row r="11" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="450" t="s">
+      <c r="A11" s="471" t="s">
         <v>117</v>
       </c>
-      <c r="B11" s="451"/>
-      <c r="C11" s="451"/>
-      <c r="D11" s="451"/>
-      <c r="E11" s="451"/>
-      <c r="F11" s="451"/>
-      <c r="G11" s="451"/>
-      <c r="H11" s="451"/>
-      <c r="I11" s="451"/>
-      <c r="J11" s="451"/>
-      <c r="K11" s="451"/>
-      <c r="L11" s="451"/>
-      <c r="M11" s="452"/>
+      <c r="B11" s="472"/>
+      <c r="C11" s="472"/>
+      <c r="D11" s="472"/>
+      <c r="E11" s="472"/>
+      <c r="F11" s="472"/>
+      <c r="G11" s="472"/>
+      <c r="H11" s="472"/>
+      <c r="I11" s="472"/>
+      <c r="J11" s="472"/>
+      <c r="K11" s="472"/>
+      <c r="L11" s="472"/>
+      <c r="M11" s="473"/>
       <c r="N11" s="303"/>
       <c r="O11" s="303"/>
       <c r="P11" s="303"/>
@@ -6874,13 +6874,13 @@
       <c r="P12" s="303"/>
     </row>
     <row r="13" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="453" t="s">
+      <c r="A13" s="474" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="454"/>
-      <c r="C13" s="454"/>
-      <c r="D13" s="454"/>
-      <c r="E13" s="454"/>
+      <c r="B13" s="475"/>
+      <c r="C13" s="475"/>
+      <c r="D13" s="475"/>
+      <c r="E13" s="475"/>
       <c r="F13" s="318"/>
       <c r="G13" s="318"/>
       <c r="H13" s="318"/>
@@ -7011,15 +7011,15 @@
       <c r="A18" s="341"/>
       <c r="B18" s="342"/>
       <c r="C18" s="342"/>
-      <c r="D18" s="445"/>
-      <c r="E18" s="445"/>
+      <c r="D18" s="466"/>
+      <c r="E18" s="466"/>
       <c r="F18" s="342"/>
       <c r="G18" s="342"/>
       <c r="H18" s="342"/>
       <c r="I18" s="343"/>
       <c r="J18" s="343"/>
-      <c r="K18" s="446"/>
-      <c r="L18" s="446"/>
+      <c r="K18" s="467"/>
+      <c r="L18" s="467"/>
       <c r="M18" s="344"/>
       <c r="N18" s="303"/>
       <c r="O18" s="345"/>
@@ -7029,18 +7029,18 @@
       <c r="A19" s="346"/>
       <c r="B19" s="347"/>
       <c r="C19" s="347"/>
-      <c r="D19" s="456" t="s">
+      <c r="D19" s="443" t="s">
         <v>73</v>
       </c>
-      <c r="E19" s="457"/>
-      <c r="F19" s="457"/>
-      <c r="G19" s="457"/>
-      <c r="H19" s="458"/>
-      <c r="I19" s="474" t="s">
+      <c r="E19" s="444"/>
+      <c r="F19" s="444"/>
+      <c r="G19" s="444"/>
+      <c r="H19" s="445"/>
+      <c r="I19" s="461" t="s">
         <v>72</v>
       </c>
-      <c r="J19" s="474"/>
-      <c r="K19" s="475"/>
+      <c r="J19" s="461"/>
+      <c r="K19" s="462"/>
       <c r="L19" s="348"/>
       <c r="M19" s="349"/>
       <c r="N19" s="303"/>
@@ -7051,11 +7051,11 @@
       <c r="A20" s="350"/>
       <c r="B20" s="295"/>
       <c r="C20" s="295"/>
-      <c r="D20" s="459"/>
-      <c r="E20" s="460"/>
-      <c r="F20" s="460"/>
-      <c r="G20" s="460"/>
-      <c r="H20" s="461"/>
+      <c r="D20" s="446"/>
+      <c r="E20" s="447"/>
+      <c r="F20" s="447"/>
+      <c r="G20" s="447"/>
+      <c r="H20" s="448"/>
       <c r="I20" s="351">
         <v>1</v>
       </c>
@@ -7127,8 +7127,8 @@
         <f>+Datos!I14</f>
         <v>0</v>
       </c>
-      <c r="L22" s="468"/>
-      <c r="M22" s="467"/>
+      <c r="L22" s="455"/>
+      <c r="M22" s="454"/>
       <c r="N22" s="303"/>
       <c r="O22" s="364"/>
       <c r="P22" s="303"/>
@@ -7158,8 +7158,8 @@
         <f>+Datos!I15</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="L23" s="466"/>
-      <c r="M23" s="467"/>
+      <c r="L23" s="453"/>
+      <c r="M23" s="454"/>
       <c r="N23" s="303"/>
       <c r="O23" s="303"/>
       <c r="P23" s="364"/>
@@ -7177,12 +7177,12 @@
       <c r="H24" s="360" t="s">
         <v>1</v>
       </c>
-      <c r="I24" s="469" t="e">
+      <c r="I24" s="456" t="e">
         <f>+Datos!G16</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="J24" s="470"/>
-      <c r="K24" s="471"/>
+      <c r="J24" s="457"/>
+      <c r="K24" s="458"/>
       <c r="L24" s="369"/>
       <c r="M24" s="362"/>
       <c r="N24" s="303"/>
@@ -7244,10 +7244,10 @@
       <c r="C28" s="386"/>
       <c r="D28" s="367"/>
       <c r="E28" s="369"/>
-      <c r="F28" s="472" t="s">
+      <c r="F28" s="459" t="s">
         <v>176</v>
       </c>
-      <c r="G28" s="473"/>
+      <c r="G28" s="460"/>
       <c r="M28" s="384"/>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.25">
@@ -7270,11 +7270,11 @@
       <c r="C30" s="386"/>
       <c r="D30" s="367"/>
       <c r="E30" s="369"/>
-      <c r="F30" s="462">
+      <c r="F30" s="449">
         <f>+Datos!E25</f>
         <v>0</v>
       </c>
-      <c r="G30" s="463"/>
+      <c r="G30" s="450"/>
       <c r="M30" s="384"/>
     </row>
     <row r="31" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -7285,11 +7285,11 @@
       <c r="C31" s="386"/>
       <c r="D31" s="367"/>
       <c r="E31" s="369"/>
-      <c r="F31" s="462">
+      <c r="F31" s="449">
         <f>+Datos!E26</f>
         <v>0</v>
       </c>
-      <c r="G31" s="463"/>
+      <c r="G31" s="450"/>
       <c r="M31" s="384"/>
     </row>
     <row r="32" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -7326,100 +7326,100 @@
       <c r="M34" s="393"/>
     </row>
     <row r="35" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="476" t="s">
+      <c r="A35" s="463" t="s">
         <v>171</v>
       </c>
-      <c r="B35" s="476"/>
-      <c r="C35" s="476"/>
-      <c r="D35" s="476"/>
-      <c r="E35" s="476"/>
-      <c r="F35" s="476"/>
-      <c r="G35" s="476"/>
-      <c r="H35" s="476"/>
-      <c r="I35" s="476"/>
-      <c r="J35" s="476"/>
-      <c r="K35" s="476"/>
-      <c r="L35" s="476"/>
-      <c r="M35" s="476"/>
-    </row>
-    <row r="36" spans="1:16" ht="34.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="465" t="s">
+      <c r="B35" s="463"/>
+      <c r="C35" s="463"/>
+      <c r="D35" s="463"/>
+      <c r="E35" s="463"/>
+      <c r="F35" s="463"/>
+      <c r="G35" s="463"/>
+      <c r="H35" s="463"/>
+      <c r="I35" s="463"/>
+      <c r="J35" s="463"/>
+      <c r="K35" s="463"/>
+      <c r="L35" s="463"/>
+      <c r="M35" s="463"/>
+    </row>
+    <row r="36" spans="1:16" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="452" t="s">
         <v>172</v>
       </c>
-      <c r="B36" s="465"/>
-      <c r="C36" s="465"/>
-      <c r="D36" s="465"/>
-      <c r="E36" s="465"/>
-      <c r="F36" s="465"/>
-      <c r="G36" s="465"/>
-      <c r="H36" s="465"/>
-      <c r="I36" s="465"/>
-      <c r="J36" s="465"/>
-      <c r="K36" s="465"/>
-      <c r="L36" s="465"/>
-      <c r="M36" s="465"/>
-    </row>
-    <row r="37" spans="1:16" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="465" t="s">
+      <c r="B36" s="452"/>
+      <c r="C36" s="452"/>
+      <c r="D36" s="452"/>
+      <c r="E36" s="452"/>
+      <c r="F36" s="452"/>
+      <c r="G36" s="452"/>
+      <c r="H36" s="452"/>
+      <c r="I36" s="452"/>
+      <c r="J36" s="452"/>
+      <c r="K36" s="452"/>
+      <c r="L36" s="452"/>
+      <c r="M36" s="452"/>
+    </row>
+    <row r="37" spans="1:16" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="452" t="s">
         <v>173</v>
       </c>
-      <c r="B37" s="465"/>
-      <c r="C37" s="465"/>
-      <c r="D37" s="465"/>
-      <c r="E37" s="465"/>
-      <c r="F37" s="465"/>
-      <c r="G37" s="465"/>
-      <c r="H37" s="465"/>
-      <c r="I37" s="465"/>
-      <c r="J37" s="465"/>
-      <c r="K37" s="465"/>
-      <c r="L37" s="465"/>
-      <c r="M37" s="465"/>
+      <c r="B37" s="452"/>
+      <c r="C37" s="452"/>
+      <c r="D37" s="452"/>
+      <c r="E37" s="452"/>
+      <c r="F37" s="452"/>
+      <c r="G37" s="452"/>
+      <c r="H37" s="452"/>
+      <c r="I37" s="452"/>
+      <c r="J37" s="452"/>
+      <c r="K37" s="452"/>
+      <c r="L37" s="452"/>
+      <c r="M37" s="452"/>
       <c r="N37" s="303"/>
       <c r="O37" s="303"/>
       <c r="P37" s="303"/>
     </row>
-    <row r="38" spans="1:16" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="465" t="s">
+    <row r="38" spans="1:16" ht="25.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="452" t="s">
         <v>174</v>
       </c>
-      <c r="B38" s="465"/>
-      <c r="C38" s="465"/>
-      <c r="D38" s="465"/>
-      <c r="E38" s="465"/>
-      <c r="F38" s="465"/>
-      <c r="G38" s="465"/>
-      <c r="H38" s="465"/>
-      <c r="I38" s="465"/>
-      <c r="J38" s="465"/>
-      <c r="K38" s="465"/>
-      <c r="L38" s="465"/>
-      <c r="M38" s="465"/>
+      <c r="B38" s="452"/>
+      <c r="C38" s="452"/>
+      <c r="D38" s="452"/>
+      <c r="E38" s="452"/>
+      <c r="F38" s="452"/>
+      <c r="G38" s="452"/>
+      <c r="H38" s="452"/>
+      <c r="I38" s="452"/>
+      <c r="J38" s="452"/>
+      <c r="K38" s="452"/>
+      <c r="L38" s="452"/>
+      <c r="M38" s="452"/>
       <c r="N38" s="303"/>
       <c r="O38" s="303"/>
       <c r="P38" s="303"/>
     </row>
     <row r="39" spans="1:16" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="464" t="s">
+      <c r="A39" s="451" t="s">
         <v>175</v>
       </c>
-      <c r="B39" s="464"/>
-      <c r="C39" s="464"/>
-      <c r="D39" s="464"/>
-      <c r="E39" s="464"/>
-      <c r="F39" s="464"/>
-      <c r="G39" s="464"/>
-      <c r="H39" s="464"/>
-      <c r="I39" s="464"/>
-      <c r="J39" s="464"/>
-      <c r="K39" s="464"/>
-      <c r="L39" s="464"/>
-      <c r="M39" s="464"/>
+      <c r="B39" s="451"/>
+      <c r="C39" s="451"/>
+      <c r="D39" s="451"/>
+      <c r="E39" s="451"/>
+      <c r="F39" s="451"/>
+      <c r="G39" s="451"/>
+      <c r="H39" s="451"/>
+      <c r="I39" s="451"/>
+      <c r="J39" s="451"/>
+      <c r="K39" s="451"/>
+      <c r="L39" s="451"/>
+      <c r="M39" s="451"/>
       <c r="N39" s="303"/>
       <c r="O39" s="303"/>
       <c r="P39" s="303"/>
     </row>
-    <row r="40" spans="1:16" ht="4.9000000000000004" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:16" ht="4.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="394"/>
       <c r="B40" s="394"/>
       <c r="C40" s="394"/>
@@ -7451,7 +7451,7 @@
       <c r="O41" s="303"/>
       <c r="P41" s="303"/>
     </row>
-    <row r="42" spans="1:16" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:16" ht="25.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="325"/>
       <c r="B42" s="325"/>
       <c r="C42" s="325"/>
@@ -7595,7 +7595,7 @@
       <c r="L49" s="295"/>
       <c r="M49" s="295"/>
     </row>
-    <row r="50" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="295"/>
       <c r="B50" s="295"/>
       <c r="C50" s="295"/>
@@ -7610,7 +7610,7 @@
       <c r="L50" s="295"/>
       <c r="M50" s="295"/>
     </row>
-    <row r="51" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="51" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="8NM1+p6p3LesDUstMxFGHu0zYxm1d4zXGYtLxhJOWwI+xJ9//NVS0q83GcKW2Ki+XgVMpMuspxvNsKuxOQLOxg==" saltValue="QYjBUm0XnOsAQh3sj8wCVA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <protectedRanges>
@@ -7619,6 +7619,17 @@
     <protectedRange sqref="C5:E6" name="Rango3_3_1_1_1_1_1_2_1_1"/>
   </protectedRanges>
   <mergeCells count="24">
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="A10:M10"/>
+    <mergeCell ref="A11:M11"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="C5:J5"/>
+    <mergeCell ref="C6:J6"/>
+    <mergeCell ref="C7:J7"/>
+    <mergeCell ref="C8:J8"/>
     <mergeCell ref="D19:H20"/>
     <mergeCell ref="F30:G30"/>
     <mergeCell ref="F31:G31"/>
@@ -7632,17 +7643,6 @@
     <mergeCell ref="A35:M35"/>
     <mergeCell ref="A36:M36"/>
     <mergeCell ref="A38:M38"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="A10:M10"/>
-    <mergeCell ref="A11:M11"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="C5:J5"/>
-    <mergeCell ref="C6:J6"/>
-    <mergeCell ref="C7:J7"/>
-    <mergeCell ref="C8:J8"/>
   </mergeCells>
   <dataValidations disablePrompts="1" count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F28:G28" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -7666,14 +7666,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:O34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.33203125" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.42578125" style="28" customWidth="1"/>
-    <col min="2" max="9" width="11.7109375" style="28" customWidth="1"/>
-    <col min="10" max="10" width="1.5703125" style="28" customWidth="1"/>
-    <col min="11" max="11" width="13.5703125" style="28" customWidth="1"/>
-    <col min="12" max="16" width="16.85546875" style="28" customWidth="1"/>
-    <col min="17" max="16384" width="10.28515625" style="28"/>
+    <col min="1" max="1" width="6.44140625" style="28" customWidth="1"/>
+    <col min="2" max="9" width="11.6640625" style="28" customWidth="1"/>
+    <col min="10" max="10" width="1.5546875" style="28" customWidth="1"/>
+    <col min="11" max="11" width="13.5546875" style="28" customWidth="1"/>
+    <col min="12" max="16" width="16.88671875" style="28" customWidth="1"/>
+    <col min="17" max="16384" width="10.33203125" style="28"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8394,7 +8394,7 @@
       <c r="J32" s="41"/>
       <c r="K32" s="41"/>
     </row>
-    <row r="33" spans="1:11" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="41"/>
       <c r="B33" s="58"/>
       <c r="C33" s="58"/>
@@ -8407,7 +8407,7 @@
       <c r="J33" s="41"/>
       <c r="K33" s="41"/>
     </row>
-    <row r="34" spans="1:11" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="30HaiR52nqiYotLJpI1mB2lORNPbDurlcC6410k5mvSvnGiAmVghg7imMzZoWOpv930Refz4w5FF+iObjCt0iQ==" saltValue="+OutNn2WwZIf1rmOnZwRlA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <protectedRanges>
@@ -8444,22 +8444,22 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:X58"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.42578125" style="15" customWidth="1"/>
-    <col min="2" max="5" width="10.42578125" style="15" customWidth="1"/>
-    <col min="6" max="8" width="13.140625" style="15" customWidth="1"/>
-    <col min="9" max="9" width="18.140625" style="15" customWidth="1"/>
-    <col min="10" max="10" width="15.42578125" style="15" customWidth="1"/>
+    <col min="1" max="1" width="19.44140625" style="15" customWidth="1"/>
+    <col min="2" max="5" width="10.44140625" style="15" customWidth="1"/>
+    <col min="6" max="8" width="13.109375" style="15" customWidth="1"/>
+    <col min="9" max="9" width="18.109375" style="15" customWidth="1"/>
+    <col min="10" max="10" width="15.44140625" style="15" customWidth="1"/>
     <col min="11" max="12" width="12" style="15" customWidth="1"/>
-    <col min="13" max="16" width="12.7109375" style="15" customWidth="1"/>
-    <col min="17" max="17" width="14.7109375" style="15" customWidth="1"/>
-    <col min="18" max="20" width="12.140625" style="15" customWidth="1"/>
+    <col min="13" max="16" width="12.6640625" style="15" customWidth="1"/>
+    <col min="17" max="17" width="14.6640625" style="15" customWidth="1"/>
+    <col min="18" max="20" width="12.109375" style="15" customWidth="1"/>
     <col min="21" max="24" width="13" style="15" customWidth="1"/>
-    <col min="25" max="16384" width="11.42578125" style="15"/>
+    <col min="25" max="16384" width="11.44140625" style="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="516"/>
       <c r="B1" s="516"/>
       <c r="C1" s="507" t="s">
@@ -8477,7 +8477,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="516"/>
       <c r="B2" s="516"/>
       <c r="C2" s="510"/>
@@ -8493,7 +8493,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="516"/>
       <c r="B3" s="516"/>
       <c r="C3" s="510"/>
@@ -8509,7 +8509,7 @@
         <v>46146</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="516"/>
       <c r="B4" s="516"/>
       <c r="C4" s="513"/>
@@ -8525,7 +8525,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="170" t="s">
         <v>50</v>
       </c>
@@ -8541,7 +8541,7 @@
       <c r="I6" s="17"/>
       <c r="J6" s="16"/>
     </row>
-    <row r="7" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="170" t="s">
         <v>49</v>
       </c>
@@ -8557,7 +8557,7 @@
       <c r="I7" s="17"/>
       <c r="J7" s="16"/>
     </row>
-    <row r="8" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="170" t="s">
         <v>48</v>
       </c>
@@ -8573,7 +8573,7 @@
       <c r="I8" s="17"/>
       <c r="J8" s="16"/>
     </row>
-    <row r="9" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="171" t="s">
         <v>161</v>
       </c>
@@ -8589,7 +8589,7 @@
       <c r="I9" s="17"/>
       <c r="J9" s="16"/>
     </row>
-    <row r="11" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="172" t="s">
         <v>168</v>
       </c>
@@ -8602,7 +8602,7 @@
       <c r="H11" s="167"/>
       <c r="I11" s="167"/>
     </row>
-    <row r="12" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="167"/>
       <c r="B12" s="167"/>
       <c r="C12" s="167"/>
@@ -8613,7 +8613,7 @@
       <c r="H12" s="167"/>
       <c r="I12" s="167"/>
     </row>
-    <row r="13" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="173" t="s">
         <v>104</v>
       </c>
@@ -8628,7 +8628,7 @@
       <c r="H13" s="167"/>
       <c r="I13" s="167"/>
     </row>
-    <row r="14" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="167"/>
       <c r="B14" s="167"/>
       <c r="C14" s="167"/>
@@ -8639,7 +8639,7 @@
       <c r="H14" s="167"/>
       <c r="I14" s="167"/>
     </row>
-    <row r="15" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="176" t="s">
         <v>108</v>
       </c>
@@ -8652,7 +8652,7 @@
       <c r="H15" s="167"/>
       <c r="I15" s="167"/>
     </row>
-    <row r="16" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="176" t="s">
         <v>109</v>
       </c>
@@ -8665,7 +8665,7 @@
       <c r="H16" s="167"/>
       <c r="I16" s="167"/>
     </row>
-    <row r="17" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="176" t="s">
         <v>110</v>
       </c>
@@ -8678,7 +8678,7 @@
       <c r="H17" s="167"/>
       <c r="I17" s="167"/>
     </row>
-    <row r="18" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="167"/>
       <c r="B18" s="167"/>
       <c r="C18" s="167"/>
@@ -8689,7 +8689,7 @@
       <c r="H18" s="167"/>
       <c r="I18" s="167"/>
     </row>
-    <row r="19" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="173" t="s">
         <v>106</v>
       </c>
@@ -8702,7 +8702,7 @@
       <c r="H19" s="167"/>
       <c r="I19" s="167"/>
     </row>
-    <row r="20" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="167"/>
       <c r="B20" s="167"/>
       <c r="C20" s="167"/>
@@ -8713,7 +8713,7 @@
       <c r="H20" s="167"/>
       <c r="I20" s="167"/>
     </row>
-    <row r="21" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="176" t="s">
         <v>111</v>
       </c>
@@ -8726,7 +8726,7 @@
       <c r="H21" s="167"/>
       <c r="I21" s="167"/>
     </row>
-    <row r="22" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="167"/>
       <c r="B22" s="167"/>
       <c r="C22" s="167"/>
@@ -8737,7 +8737,7 @@
       <c r="H22" s="167"/>
       <c r="I22" s="167"/>
     </row>
-    <row r="23" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="172" t="s">
         <v>107</v>
       </c>
@@ -8750,7 +8750,7 @@
       <c r="H23" s="167"/>
       <c r="I23" s="167"/>
     </row>
-    <row r="24" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="167"/>
       <c r="B24" s="167"/>
       <c r="C24" s="167"/>
@@ -8761,11 +8761,11 @@
       <c r="H24" s="167"/>
       <c r="I24" s="167"/>
     </row>
-    <row r="25" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="26" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="27" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="28" spans="1:24" ht="54.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="29" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:24" ht="54.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F29" s="91"/>
       <c r="H29" s="91"/>
       <c r="I29" s="91"/>
@@ -8780,7 +8780,7 @@
       <c r="T29" s="167"/>
       <c r="U29" s="167"/>
     </row>
-    <row r="30" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L30" s="166"/>
       <c r="M30" s="167"/>
       <c r="N30" s="167"/>
@@ -8792,7 +8792,7 @@
       <c r="T30" s="167"/>
       <c r="U30" s="167"/>
     </row>
-    <row r="31" spans="1:24" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:24" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="L31" s="168"/>
       <c r="M31" s="168"/>
       <c r="N31" s="168"/>
@@ -8804,7 +8804,7 @@
       <c r="T31" s="168"/>
       <c r="U31" s="168"/>
     </row>
-    <row r="32" spans="1:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="139" t="s">
         <v>47</v>
       </c>
@@ -8878,7 +8878,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="33" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="126" t="s">
         <v>59</v>
       </c>
@@ -8919,7 +8919,7 @@
       <c r="W33" s="112"/>
       <c r="X33" s="128"/>
     </row>
-    <row r="34" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="122" t="s">
         <v>64</v>
       </c>
@@ -8999,7 +8999,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="35" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="124" t="s">
         <v>60</v>
       </c>
@@ -9073,7 +9073,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="36" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="122" t="s">
         <v>65</v>
       </c>
@@ -9153,7 +9153,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="37" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="124" t="s">
         <v>60</v>
       </c>
@@ -9370,7 +9370,7 @@
       <c r="W40" s="137"/>
       <c r="X40" s="137"/>
     </row>
-    <row r="41" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="111"/>
       <c r="D41" s="111"/>
       <c r="E41" s="111"/>
@@ -9380,7 +9380,7 @@
       <c r="I41" s="111"/>
       <c r="J41" s="111"/>
     </row>
-    <row r="42" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="111"/>
       <c r="B42" s="14"/>
       <c r="C42" s="13"/>
@@ -9392,7 +9392,7 @@
       <c r="I42" s="111"/>
       <c r="J42" s="111"/>
     </row>
-    <row r="43" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="148"/>
       <c r="B43" s="152" t="str">
         <f>A34</f>
@@ -9413,7 +9413,7 @@
       <c r="I43" s="111"/>
       <c r="J43" s="111"/>
     </row>
-    <row r="44" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="148"/>
       <c r="B44" s="152" t="str">
         <f>A36</f>
@@ -9434,7 +9434,7 @@
       <c r="I44" s="111"/>
       <c r="J44" s="111"/>
     </row>
-    <row r="45" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="152" t="str">
         <f>A38</f>
         <v>factor de presición</v>
@@ -9454,7 +9454,7 @@
       <c r="I45" s="111"/>
       <c r="J45" s="111"/>
     </row>
-    <row r="46" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="505"/>
       <c r="B46" s="506"/>
       <c r="C46" s="151" t="e">
@@ -9469,7 +9469,7 @@
       <c r="I46" s="111"/>
       <c r="J46" s="111"/>
     </row>
-    <row r="47" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A47" s="111"/>
       <c r="B47" s="111"/>
       <c r="C47" s="111"/>
@@ -9481,7 +9481,7 @@
       <c r="I47" s="111"/>
       <c r="J47" s="111"/>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="290" t="s">
         <v>162</v>
       </c>
@@ -9499,7 +9499,7 @@
       </c>
       <c r="H55" s="521"/>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="167"/>
       <c r="B56" s="167"/>
       <c r="C56" s="167"/>
@@ -9509,7 +9509,7 @@
       <c r="G56" s="167"/>
       <c r="H56" s="167"/>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="287" t="s">
         <v>166</v>
       </c>
@@ -9527,7 +9527,7 @@
       </c>
       <c r="H57" s="503"/>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="167"/>
       <c r="B58" s="167"/>
       <c r="C58" s="167"/>
@@ -9562,24 +9562,24 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A2:G30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" style="15"/>
-    <col min="2" max="2" width="13.5703125" style="15" customWidth="1"/>
+    <col min="1" max="1" width="11.44140625" style="15"/>
+    <col min="2" max="2" width="13.5546875" style="15" customWidth="1"/>
     <col min="3" max="3" width="12" style="15" customWidth="1"/>
-    <col min="4" max="6" width="11.42578125" style="15"/>
-    <col min="7" max="7" width="14.42578125" style="15" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" style="15"/>
-    <col min="9" max="9" width="11.85546875" style="15" customWidth="1"/>
-    <col min="10" max="16384" width="11.42578125" style="15"/>
+    <col min="4" max="6" width="11.44140625" style="15"/>
+    <col min="7" max="7" width="14.44140625" style="15" customWidth="1"/>
+    <col min="8" max="8" width="11.44140625" style="15"/>
+    <col min="9" max="9" width="11.88671875" style="15" customWidth="1"/>
+    <col min="10" max="16384" width="11.44140625" style="15"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="100" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B4" s="101" t="str">
         <f>+Datos!B13</f>
         <v>Lectura de la arcilla</v>
@@ -9597,7 +9597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B5" s="101" t="str">
         <f>+Datos!B14</f>
         <v>Lectura de la arena</v>
@@ -9615,7 +9615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="523" t="s">
         <v>58</v>
       </c>
@@ -9625,14 +9625,14 @@
       <c r="E9" s="26"/>
       <c r="F9" s="26"/>
     </row>
-    <row r="10" spans="1:7" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="21"/>
       <c r="C10" s="21"/>
       <c r="D10" s="21"/>
       <c r="E10" s="27"/>
       <c r="F10" s="94"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="102" t="s">
         <v>98</v>
       </c>
@@ -9640,13 +9640,13 @@
       <c r="F11" s="94"/>
       <c r="G11" s="94"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="103"/>
       <c r="B12" s="91"/>
       <c r="F12" s="94"/>
       <c r="G12" s="94"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="104">
         <v>1</v>
       </c>
@@ -9657,7 +9657,7 @@
         <v>381.6</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="104">
         <v>2</v>
       </c>
@@ -9671,7 +9671,7 @@
       <c r="F14" s="95"/>
       <c r="G14" s="95"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="104">
         <v>3</v>
       </c>
@@ -9685,7 +9685,7 @@
       <c r="F15" s="95"/>
       <c r="G15" s="95"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="104">
         <v>4</v>
       </c>
@@ -9694,7 +9694,7 @@
       <c r="F16" s="95"/>
       <c r="G16" s="95"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="525" t="s">
         <v>96</v>
       </c>
@@ -9704,7 +9704,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="525"/>
       <c r="B18" s="525"/>
       <c r="C18" s="108">
@@ -9714,7 +9714,7 @@
       <c r="F18" s="95"/>
       <c r="G18" s="95"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="20"/>
       <c r="B19" s="21"/>
       <c r="C19" s="21"/>
@@ -9722,66 +9722,66 @@
       <c r="F19" s="95"/>
       <c r="G19" s="95"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B20" s="21"/>
       <c r="C20" s="21"/>
       <c r="D20" s="21"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="504"/>
       <c r="B21" s="21"/>
       <c r="C21" s="21"/>
       <c r="D21" s="21"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="504"/>
       <c r="B22" s="21"/>
       <c r="C22" s="21"/>
       <c r="D22" s="21"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="504"/>
       <c r="B23" s="21"/>
       <c r="C23" s="21"/>
       <c r="D23" s="21"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="504"/>
       <c r="B24" s="21"/>
       <c r="C24" s="21"/>
       <c r="D24" s="21"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="522"/>
       <c r="B25" s="21"/>
       <c r="C25" s="21"/>
       <c r="D25" s="21"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="522"/>
       <c r="B26" s="21"/>
       <c r="C26" s="21"/>
       <c r="D26" s="21"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="522"/>
       <c r="B27" s="21"/>
       <c r="C27" s="21"/>
       <c r="D27" s="21"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="522"/>
       <c r="B28" s="21"/>
       <c r="C28" s="21"/>
       <c r="D28" s="21"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="20"/>
       <c r="B29" s="22"/>
       <c r="C29" s="23"/>
       <c r="D29" s="22"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C30" s="24"/>
       <c r="D30" s="25"/>
     </row>
@@ -9801,30 +9801,30 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="39.7109375" style="186" customWidth="1"/>
-    <col min="2" max="16384" width="11.5703125" style="186"/>
+    <col min="1" max="1" width="39.6640625" style="186" customWidth="1"/>
+    <col min="2" max="16384" width="11.5546875" style="186"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="9.6" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="9.6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="187"/>
     </row>
-    <row r="3" spans="1:11" ht="6.6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="3" spans="1:11" ht="6.6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="292" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="93"/>
       <c r="H5" s="188"/>
       <c r="I5" s="526"/>
       <c r="J5" s="526"/>
       <c r="K5" s="526"/>
     </row>
-    <row r="6" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="93" t="s">
         <v>94</v>
       </c>
@@ -9836,7 +9836,7 @@
       <c r="J6" s="191"/>
       <c r="K6" s="191"/>
     </row>
-    <row r="7" spans="1:11" ht="7.9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" ht="7.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="93"/>
       <c r="B7" s="192"/>
       <c r="H7" s="288"/>
@@ -9844,7 +9844,7 @@
       <c r="J7" s="191"/>
       <c r="K7" s="191"/>
     </row>
-    <row r="8" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="193" t="s">
         <v>120</v>
       </c>
@@ -9855,7 +9855,7 @@
       <c r="D8" s="527"/>
       <c r="E8" s="92"/>
     </row>
-    <row r="9" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="193" t="s">
         <v>121</v>
       </c>
@@ -9882,18 +9882,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr codeName="Hoja3"/>
   <dimension ref="A2:M9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="10.42578125" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" customWidth="1"/>
+    <col min="1" max="2" width="10.44140625" customWidth="1"/>
+    <col min="3" max="3" width="18.33203125" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" customWidth="1"/>
-    <col min="11" max="11" width="17.7109375" customWidth="1"/>
-    <col min="12" max="12" width="12.42578125" customWidth="1"/>
-    <col min="13" max="13" width="15.42578125" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" customWidth="1"/>
+    <col min="11" max="11" width="17.6640625" customWidth="1"/>
+    <col min="12" max="12" width="12.44140625" customWidth="1"/>
+    <col min="13" max="13" width="15.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="528" t="s">
         <v>11</v>
       </c>
@@ -9932,7 +9932,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7">
         <v>4400</v>
       </c>
@@ -9978,7 +9978,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="6" t="str">
@@ -10015,7 +10015,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <f>+B3+1</f>
         <v>4402</v>
@@ -10058,7 +10058,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="6" t="str">
@@ -10095,7 +10095,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <f>+B5+1</f>
         <v>4404</v>
@@ -10138,7 +10138,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="6" t="str">
@@ -10175,7 +10175,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:B2"/>

</xml_diff>

<commit_message>
feat(templates): migrate and update all soils and aggregates excel templates to production folders
</commit_message>
<xml_diff>
--- a/app/templates/informes/EquiArena/1-INF.-N-000-26-SU21-E.-ARENA-V08.xlsx
+++ b/app/templates/informes/EquiArena/1-INF.-N-000-26-SU21-E.-ARENA-V08.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\informes\EquiArena\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\3.0 Formatos e informes\2026\1.0 Informe de ensayo\1.1 Informe Suelo\INFORME ACREDITADO-E ISO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B33F4E50-C0BB-4C21-BAEE-5C0C7EE2931B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C4813B6-51FD-4DEF-91D9-7E6E91CFE9AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="556" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="556" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FORMATO" sheetId="97" r:id="rId1"/>
@@ -2945,6 +2945,123 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="178" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="44" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="44" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="44" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="1"/>
@@ -2973,121 +3090,46 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="18" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="44" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="44" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="44" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="178" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3156,48 +3198,6 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="18" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4648,7 +4648,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -4707,7 +4707,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="datos de ecuacion del anillo"/>
@@ -4826,7 +4826,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -4877,7 +4877,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -4929,7 +4929,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink5.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="BGA"/>
@@ -4961,7 +4961,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink6.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -5666,23 +5666,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0883903-CEA4-449A-A5F8-47E41E2F4676}">
   <dimension ref="A1:N56"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.33203125" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.28515625" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.88671875" style="199" customWidth="1"/>
-    <col min="2" max="2" width="9.109375" style="199" customWidth="1"/>
-    <col min="3" max="3" width="5.6640625" style="199" customWidth="1"/>
-    <col min="4" max="4" width="10.109375" style="199" customWidth="1"/>
-    <col min="5" max="5" width="8.109375" style="199" customWidth="1"/>
-    <col min="6" max="6" width="11.33203125" style="199" customWidth="1"/>
-    <col min="7" max="7" width="11.109375" style="199" customWidth="1"/>
+    <col min="1" max="1" width="6.85546875" style="199" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="199" customWidth="1"/>
+    <col min="3" max="3" width="5.7109375" style="199" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" style="199" customWidth="1"/>
+    <col min="5" max="5" width="8.140625" style="199" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" style="199" customWidth="1"/>
+    <col min="7" max="7" width="11.140625" style="199" customWidth="1"/>
     <col min="8" max="10" width="13" style="199" customWidth="1"/>
-    <col min="11" max="11" width="6.44140625" style="199" customWidth="1"/>
-    <col min="12" max="12" width="9.44140625" style="199" customWidth="1"/>
-    <col min="13" max="14" width="10.6640625" style="199" customWidth="1"/>
-    <col min="15" max="16384" width="10.33203125" style="199"/>
+    <col min="11" max="11" width="6.42578125" style="199" customWidth="1"/>
+    <col min="12" max="12" width="9.42578125" style="199" customWidth="1"/>
+    <col min="13" max="14" width="10.7109375" style="199" customWidth="1"/>
+    <col min="15" max="16384" width="10.28515625" style="199"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A1" s="195"/>
       <c r="B1" s="196"/>
       <c r="C1" s="196"/>
@@ -5694,7 +5694,7 @@
       <c r="I1" s="197"/>
       <c r="J1" s="198"/>
     </row>
-    <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="200"/>
       <c r="B2" s="201"/>
       <c r="C2" s="201"/>
@@ -5710,7 +5710,7 @@
       </c>
       <c r="N2" s="280"/>
     </row>
-    <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="200"/>
       <c r="B3" s="201"/>
       <c r="C3" s="201"/>
@@ -5726,7 +5726,7 @@
       </c>
       <c r="N3" s="281"/>
     </row>
-    <row r="4" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="200"/>
       <c r="B4" s="201"/>
       <c r="C4" s="201"/>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="N4" s="281"/>
     </row>
-    <row r="5" spans="1:14" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="204"/>
       <c r="B5" s="205"/>
       <c r="C5" s="205"/>
@@ -5758,7 +5758,7 @@
       </c>
       <c r="N5" s="281"/>
     </row>
-    <row r="6" spans="1:14" ht="5.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="5.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A6" s="207"/>
       <c r="B6" s="207"/>
       <c r="C6" s="207"/>
@@ -5772,43 +5772,43 @@
       <c r="M6" s="282"/>
       <c r="N6" s="283"/>
     </row>
-    <row r="7" spans="1:14" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="437" t="s">
+    <row r="7" spans="1:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="409" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="437"/>
-      <c r="C7" s="437"/>
-      <c r="D7" s="437"/>
-      <c r="E7" s="437"/>
-      <c r="F7" s="437"/>
-      <c r="G7" s="437"/>
-      <c r="H7" s="437"/>
-      <c r="I7" s="437"/>
-      <c r="J7" s="437"/>
+      <c r="B7" s="409"/>
+      <c r="C7" s="409"/>
+      <c r="D7" s="409"/>
+      <c r="E7" s="409"/>
+      <c r="F7" s="409"/>
+      <c r="G7" s="409"/>
+      <c r="H7" s="409"/>
+      <c r="I7" s="409"/>
+      <c r="J7" s="409"/>
       <c r="M7" s="279" t="s">
         <v>119</v>
       </c>
       <c r="N7" s="283"/>
     </row>
-    <row r="8" spans="1:14" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="438" t="s">
+    <row r="8" spans="1:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="410" t="s">
         <v>122</v>
       </c>
-      <c r="B8" s="438"/>
-      <c r="C8" s="438"/>
-      <c r="D8" s="438"/>
-      <c r="E8" s="438"/>
-      <c r="F8" s="438"/>
-      <c r="G8" s="438"/>
-      <c r="H8" s="438"/>
-      <c r="I8" s="438"/>
-      <c r="J8" s="438"/>
+      <c r="B8" s="410"/>
+      <c r="C8" s="410"/>
+      <c r="D8" s="410"/>
+      <c r="E8" s="410"/>
+      <c r="F8" s="410"/>
+      <c r="G8" s="410"/>
+      <c r="H8" s="410"/>
+      <c r="I8" s="410"/>
+      <c r="J8" s="410"/>
       <c r="M8" s="279" t="s">
         <v>157</v>
       </c>
       <c r="N8" s="284"/>
     </row>
-    <row r="9" spans="1:14" ht="6.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="6.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="208"/>
       <c r="B9" s="208"/>
       <c r="C9" s="208"/>
@@ -5824,39 +5824,39 @@
       </c>
       <c r="N9" s="283"/>
     </row>
-    <row r="10" spans="1:14" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="439" t="s">
+    <row r="10" spans="1:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="411" t="s">
         <v>123</v>
       </c>
-      <c r="C10" s="439"/>
-      <c r="D10" s="439" t="s">
+      <c r="C10" s="411"/>
+      <c r="D10" s="411" t="s">
         <v>124</v>
       </c>
-      <c r="E10" s="439"/>
-      <c r="F10" s="439" t="s">
+      <c r="E10" s="411"/>
+      <c r="F10" s="411" t="s">
         <v>125</v>
       </c>
-      <c r="G10" s="439"/>
-      <c r="H10" s="439" t="s">
+      <c r="G10" s="411"/>
+      <c r="H10" s="411" t="s">
         <v>126</v>
       </c>
-      <c r="I10" s="439"/>
+      <c r="I10" s="411"/>
       <c r="J10" s="209"/>
       <c r="K10" s="210"/>
       <c r="L10" s="210"/>
       <c r="M10" s="282"/>
       <c r="N10" s="283"/>
     </row>
-    <row r="11" spans="1:14" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="211"/>
-      <c r="B11" s="439"/>
-      <c r="C11" s="439"/>
-      <c r="D11" s="439"/>
-      <c r="E11" s="439"/>
-      <c r="F11" s="439"/>
-      <c r="G11" s="439"/>
-      <c r="H11" s="439"/>
-      <c r="I11" s="439"/>
+      <c r="B11" s="411"/>
+      <c r="C11" s="411"/>
+      <c r="D11" s="411"/>
+      <c r="E11" s="411"/>
+      <c r="F11" s="411"/>
+      <c r="G11" s="411"/>
+      <c r="H11" s="411"/>
+      <c r="I11" s="411"/>
       <c r="J11" s="212"/>
       <c r="K11" s="210"/>
       <c r="L11" s="210"/>
@@ -5865,7 +5865,7 @@
       </c>
       <c r="N11" s="283"/>
     </row>
-    <row r="12" spans="1:14" ht="7.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" ht="7.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="211"/>
       <c r="B12" s="211"/>
       <c r="C12" s="213"/>
@@ -5883,19 +5883,19 @@
       </c>
       <c r="N12" s="284"/>
     </row>
-    <row r="13" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="440" t="s">
+    <row r="13" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="412" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="441"/>
-      <c r="C13" s="441"/>
-      <c r="D13" s="441"/>
-      <c r="E13" s="441"/>
-      <c r="F13" s="441"/>
-      <c r="G13" s="441"/>
-      <c r="H13" s="441"/>
-      <c r="I13" s="441"/>
-      <c r="J13" s="442"/>
+      <c r="B13" s="413"/>
+      <c r="C13" s="413"/>
+      <c r="D13" s="413"/>
+      <c r="E13" s="413"/>
+      <c r="F13" s="413"/>
+      <c r="G13" s="413"/>
+      <c r="H13" s="413"/>
+      <c r="I13" s="413"/>
+      <c r="J13" s="414"/>
       <c r="K13" s="210"/>
       <c r="L13" s="210"/>
       <c r="M13" s="279" t="s">
@@ -5903,25 +5903,25 @@
       </c>
       <c r="N13" s="284"/>
     </row>
-    <row r="14" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="434" t="s">
+    <row r="14" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="406" t="s">
         <v>117</v>
       </c>
-      <c r="B14" s="435"/>
-      <c r="C14" s="435"/>
-      <c r="D14" s="435"/>
-      <c r="E14" s="435"/>
-      <c r="F14" s="435"/>
-      <c r="G14" s="435"/>
-      <c r="H14" s="435"/>
-      <c r="I14" s="435"/>
-      <c r="J14" s="436"/>
+      <c r="B14" s="407"/>
+      <c r="C14" s="407"/>
+      <c r="D14" s="407"/>
+      <c r="E14" s="407"/>
+      <c r="F14" s="407"/>
+      <c r="G14" s="407"/>
+      <c r="H14" s="407"/>
+      <c r="I14" s="407"/>
+      <c r="J14" s="408"/>
       <c r="K14" s="210"/>
       <c r="L14" s="210"/>
       <c r="M14" s="282"/>
       <c r="N14" s="283"/>
     </row>
-    <row r="15" spans="1:14" ht="6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" ht="6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="216"/>
       <c r="B15" s="217"/>
       <c r="C15" s="218"/>
@@ -5939,23 +5939,23 @@
       </c>
       <c r="N15" s="285"/>
     </row>
-    <row r="16" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="221"/>
-      <c r="B16" s="426" t="s">
+      <c r="B16" s="415" t="s">
         <v>118</v>
       </c>
-      <c r="C16" s="426"/>
-      <c r="D16" s="426"/>
+      <c r="C16" s="415"/>
+      <c r="D16" s="415"/>
       <c r="E16" s="222"/>
-      <c r="F16" s="427" t="s">
+      <c r="F16" s="416" t="s">
         <v>127</v>
       </c>
-      <c r="G16" s="427"/>
+      <c r="G16" s="416"/>
       <c r="H16" s="222"/>
-      <c r="I16" s="428" t="s">
+      <c r="I16" s="417" t="s">
         <v>128</v>
       </c>
-      <c r="J16" s="431"/>
+      <c r="J16" s="420"/>
       <c r="K16" s="210"/>
       <c r="L16" s="210"/>
       <c r="M16" s="279" t="s">
@@ -5963,17 +5963,17 @@
       </c>
       <c r="N16" s="285"/>
     </row>
-    <row r="17" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="221"/>
-      <c r="B17" s="417"/>
-      <c r="C17" s="418"/>
-      <c r="D17" s="419"/>
+      <c r="B17" s="423"/>
+      <c r="C17" s="424"/>
+      <c r="D17" s="425"/>
       <c r="E17" s="223"/>
-      <c r="F17" s="417"/>
-      <c r="G17" s="419"/>
+      <c r="F17" s="423"/>
+      <c r="G17" s="425"/>
       <c r="H17" s="222"/>
-      <c r="I17" s="429"/>
-      <c r="J17" s="432"/>
+      <c r="I17" s="418"/>
+      <c r="J17" s="421"/>
       <c r="K17" s="210"/>
       <c r="L17" s="210"/>
       <c r="M17" s="279" t="s">
@@ -5981,17 +5981,17 @@
       </c>
       <c r="N17" s="286"/>
     </row>
-    <row r="18" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E18" s="223"/>
       <c r="F18" s="223"/>
       <c r="G18" s="223"/>
       <c r="H18" s="222"/>
-      <c r="I18" s="430"/>
-      <c r="J18" s="433"/>
+      <c r="I18" s="419"/>
+      <c r="J18" s="422"/>
       <c r="L18" s="210"/>
       <c r="M18" s="224"/>
     </row>
-    <row r="19" spans="1:14" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="225"/>
       <c r="B19" s="223"/>
       <c r="C19" s="223"/>
@@ -6005,13 +6005,13 @@
       <c r="L19" s="210"/>
       <c r="M19" s="224"/>
     </row>
-    <row r="20" spans="1:14" s="228" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" s="228" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="227"/>
-      <c r="B20" s="413" t="s">
+      <c r="B20" s="426" t="s">
         <v>129</v>
       </c>
-      <c r="C20" s="413"/>
-      <c r="D20" s="415"/>
+      <c r="C20" s="426"/>
+      <c r="D20" s="428"/>
       <c r="F20" s="229" t="s">
         <v>130</v>
       </c>
@@ -6022,20 +6022,20 @@
       <c r="L20" s="231"/>
       <c r="M20" s="224"/>
     </row>
-    <row r="21" spans="1:14" s="228" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" s="228" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="232"/>
-      <c r="B21" s="414"/>
-      <c r="C21" s="414"/>
-      <c r="D21" s="416"/>
-      <c r="F21" s="417"/>
-      <c r="G21" s="418"/>
-      <c r="H21" s="419"/>
+      <c r="B21" s="427"/>
+      <c r="C21" s="427"/>
+      <c r="D21" s="429"/>
+      <c r="F21" s="423"/>
+      <c r="G21" s="424"/>
+      <c r="H21" s="425"/>
       <c r="I21" s="230"/>
       <c r="J21" s="226"/>
       <c r="L21" s="231"/>
       <c r="M21" s="224"/>
     </row>
-    <row r="22" spans="1:14" s="228" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" s="228" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="232"/>
       <c r="B22" s="230"/>
       <c r="C22" s="230"/>
@@ -6045,7 +6045,7 @@
       <c r="L22" s="231"/>
       <c r="M22" s="224"/>
     </row>
-    <row r="23" spans="1:14" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="233"/>
       <c r="B23" s="234"/>
       <c r="C23" s="234"/>
@@ -6058,14 +6058,14 @@
       <c r="J23" s="235"/>
       <c r="L23" s="236"/>
     </row>
-    <row r="24" spans="1:14" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="67"/>
       <c r="B24" s="67"/>
       <c r="J24" s="67"/>
       <c r="K24" s="210"/>
       <c r="L24" s="237"/>
     </row>
-    <row r="25" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="238" t="s">
         <v>131</v>
       </c>
@@ -6089,7 +6089,7 @@
       <c r="K25" s="244"/>
       <c r="L25" s="245"/>
     </row>
-    <row r="26" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="246" t="s">
         <v>135</v>
       </c>
@@ -6109,7 +6109,7 @@
       <c r="K26" s="252"/>
       <c r="N26" s="253"/>
     </row>
-    <row r="27" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="246" t="s">
         <v>136</v>
       </c>
@@ -6129,7 +6129,7 @@
       <c r="K27" s="255"/>
       <c r="L27" s="253"/>
     </row>
-    <row r="28" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="246" t="s">
         <v>138</v>
       </c>
@@ -6149,7 +6149,7 @@
       <c r="K28" s="257"/>
       <c r="L28" s="253"/>
     </row>
-    <row r="29" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="246" t="s">
         <v>139</v>
       </c>
@@ -6169,7 +6169,7 @@
       <c r="K29" s="257"/>
       <c r="L29" s="236"/>
     </row>
-    <row r="30" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="246" t="s">
         <v>14</v>
       </c>
@@ -6189,7 +6189,7 @@
       <c r="K30" s="257"/>
       <c r="L30" s="210"/>
     </row>
-    <row r="31" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="246" t="s">
         <v>15</v>
       </c>
@@ -6209,7 +6209,7 @@
       <c r="K31" s="257"/>
       <c r="L31" s="210"/>
     </row>
-    <row r="32" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="246" t="s">
         <v>140</v>
       </c>
@@ -6229,7 +6229,7 @@
       <c r="K32" s="258"/>
       <c r="L32" s="210"/>
     </row>
-    <row r="33" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="246" t="s">
         <v>141</v>
       </c>
@@ -6249,7 +6249,7 @@
       <c r="K33" s="262"/>
       <c r="L33" s="210"/>
     </row>
-    <row r="34" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="246" t="s">
         <v>142</v>
       </c>
@@ -6269,7 +6269,7 @@
       <c r="K34" s="264"/>
       <c r="L34" s="210"/>
     </row>
-    <row r="35" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="246" t="s">
         <v>143</v>
       </c>
@@ -6289,7 +6289,7 @@
       <c r="K35" s="210"/>
       <c r="L35" s="210"/>
     </row>
-    <row r="36" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="246" t="s">
         <v>145</v>
       </c>
@@ -6303,15 +6303,15 @@
       <c r="G36" s="250" t="s">
         <v>1</v>
       </c>
-      <c r="H36" s="420">
+      <c r="H36" s="430">
         <v>31</v>
       </c>
-      <c r="I36" s="421"/>
-      <c r="J36" s="422"/>
+      <c r="I36" s="431"/>
+      <c r="J36" s="432"/>
       <c r="K36" s="210"/>
       <c r="L36" s="210"/>
     </row>
-    <row r="37" spans="1:12" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:12" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="267"/>
       <c r="B37" s="267"/>
       <c r="C37" s="268"/>
@@ -6325,16 +6325,16 @@
       <c r="K37" s="210"/>
       <c r="L37" s="210"/>
     </row>
-    <row r="38" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="423" t="s">
+    <row r="38" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="433" t="s">
         <v>146</v>
       </c>
-      <c r="B38" s="424"/>
-      <c r="C38" s="425"/>
-      <c r="D38" s="423" t="s">
+      <c r="B38" s="434"/>
+      <c r="C38" s="435"/>
+      <c r="D38" s="433" t="s">
         <v>147</v>
       </c>
-      <c r="E38" s="425"/>
+      <c r="E38" s="435"/>
       <c r="F38" s="271" t="s">
         <v>100</v>
       </c>
@@ -6345,14 +6345,14 @@
       <c r="K38" s="210"/>
       <c r="L38" s="210"/>
     </row>
-    <row r="39" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="406" t="s">
+    <row r="39" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="436" t="s">
         <v>148</v>
       </c>
-      <c r="B39" s="407"/>
-      <c r="C39" s="408"/>
-      <c r="D39" s="406"/>
-      <c r="E39" s="408"/>
+      <c r="B39" s="437"/>
+      <c r="C39" s="438"/>
+      <c r="D39" s="436"/>
+      <c r="E39" s="438"/>
       <c r="F39" s="233"/>
       <c r="G39" s="234"/>
       <c r="H39" s="234"/>
@@ -6361,14 +6361,14 @@
       <c r="K39" s="210"/>
       <c r="L39" s="210"/>
     </row>
-    <row r="40" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="406" t="s">
+    <row r="40" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="436" t="s">
         <v>149</v>
       </c>
-      <c r="B40" s="407"/>
-      <c r="C40" s="408"/>
-      <c r="D40" s="406"/>
-      <c r="E40" s="408"/>
+      <c r="B40" s="437"/>
+      <c r="C40" s="438"/>
+      <c r="D40" s="436"/>
+      <c r="E40" s="438"/>
       <c r="F40" s="274"/>
       <c r="G40" s="272"/>
       <c r="H40" s="272"/>
@@ -6377,67 +6377,67 @@
       <c r="K40" s="210"/>
       <c r="L40" s="210"/>
     </row>
-    <row r="41" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="406" t="s">
+    <row r="41" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="436" t="s">
         <v>150</v>
       </c>
-      <c r="B41" s="407"/>
-      <c r="C41" s="408"/>
-      <c r="D41" s="406"/>
-      <c r="E41" s="408"/>
+      <c r="B41" s="437"/>
+      <c r="C41" s="438"/>
+      <c r="D41" s="436"/>
+      <c r="E41" s="438"/>
       <c r="F41" s="221"/>
       <c r="K41" s="210"/>
       <c r="L41" s="210"/>
     </row>
-    <row r="42" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="410" t="s">
+    <row r="42" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="440" t="s">
         <v>151</v>
       </c>
-      <c r="B42" s="411"/>
-      <c r="C42" s="412"/>
-      <c r="D42" s="406"/>
-      <c r="E42" s="408"/>
+      <c r="B42" s="441"/>
+      <c r="C42" s="442"/>
+      <c r="D42" s="436"/>
+      <c r="E42" s="438"/>
       <c r="F42" s="221"/>
       <c r="K42" s="210"/>
       <c r="L42" s="210"/>
     </row>
-    <row r="43" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="410" t="s">
+    <row r="43" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="440" t="s">
         <v>152</v>
       </c>
-      <c r="B43" s="411"/>
-      <c r="C43" s="412"/>
-      <c r="D43" s="406"/>
-      <c r="E43" s="408"/>
+      <c r="B43" s="441"/>
+      <c r="C43" s="442"/>
+      <c r="D43" s="436"/>
+      <c r="E43" s="438"/>
       <c r="F43" s="221"/>
       <c r="K43" s="210"/>
       <c r="L43" s="210"/>
     </row>
-    <row r="44" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="406" t="s">
+    <row r="44" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="436" t="s">
         <v>153</v>
       </c>
-      <c r="B44" s="407"/>
-      <c r="C44" s="408"/>
-      <c r="D44" s="406"/>
-      <c r="E44" s="408"/>
+      <c r="B44" s="437"/>
+      <c r="C44" s="438"/>
+      <c r="D44" s="436"/>
+      <c r="E44" s="438"/>
       <c r="F44" s="221"/>
       <c r="K44" s="210"/>
       <c r="L44" s="210"/>
     </row>
-    <row r="45" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="406" t="s">
+    <row r="45" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="436" t="s">
         <v>154</v>
       </c>
-      <c r="B45" s="407"/>
-      <c r="C45" s="408"/>
-      <c r="D45" s="406"/>
-      <c r="E45" s="408"/>
+      <c r="B45" s="437"/>
+      <c r="C45" s="438"/>
+      <c r="D45" s="436"/>
+      <c r="E45" s="438"/>
       <c r="F45" s="221"/>
       <c r="K45" s="210"/>
       <c r="L45" s="210"/>
     </row>
-    <row r="46" spans="1:12" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:12" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="275"/>
       <c r="B46" s="275"/>
       <c r="C46" s="270"/>
@@ -6451,7 +6451,7 @@
       <c r="K46" s="210"/>
       <c r="L46" s="210"/>
     </row>
-    <row r="47" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="276"/>
       <c r="B47" s="276"/>
       <c r="C47" s="270"/>
@@ -6459,7 +6459,7 @@
       <c r="K47" s="210"/>
       <c r="L47" s="210"/>
     </row>
-    <row r="48" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="276"/>
       <c r="B48" s="276"/>
       <c r="C48" s="270"/>
@@ -6467,7 +6467,7 @@
       <c r="K48" s="210"/>
       <c r="L48" s="210"/>
     </row>
-    <row r="49" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="276"/>
       <c r="B49" s="276"/>
       <c r="C49" s="270"/>
@@ -6475,7 +6475,7 @@
       <c r="K49" s="210"/>
       <c r="L49" s="210"/>
     </row>
-    <row r="50" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="277"/>
       <c r="B50" s="277"/>
       <c r="C50" s="270"/>
@@ -6489,7 +6489,7 @@
       <c r="K50" s="210"/>
       <c r="L50" s="210"/>
     </row>
-    <row r="51" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="278" t="s">
         <v>18</v>
       </c>
@@ -6505,7 +6505,7 @@
       <c r="K51" s="210"/>
       <c r="L51" s="210"/>
     </row>
-    <row r="52" spans="1:12" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="278" t="s">
         <v>155</v>
       </c>
@@ -6523,23 +6523,23 @@
       <c r="K52" s="210"/>
       <c r="L52" s="210"/>
     </row>
-    <row r="53" spans="1:12" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="409" t="s">
+    <row r="53" spans="1:12" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="54" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="439" t="s">
         <v>170</v>
       </c>
-      <c r="B54" s="409"/>
-      <c r="C54" s="409"/>
-      <c r="D54" s="409"/>
-      <c r="E54" s="409"/>
-      <c r="F54" s="409"/>
-      <c r="G54" s="409"/>
-      <c r="H54" s="409"/>
-      <c r="I54" s="409"/>
-      <c r="J54" s="409"/>
-    </row>
-    <row r="55" spans="1:12" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="1:12" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="B54" s="439"/>
+      <c r="C54" s="439"/>
+      <c r="D54" s="439"/>
+      <c r="E54" s="439"/>
+      <c r="F54" s="439"/>
+      <c r="G54" s="439"/>
+      <c r="H54" s="439"/>
+      <c r="I54" s="439"/>
+      <c r="J54" s="439"/>
+    </row>
+    <row r="55" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="56" spans="1:12" ht="15.95" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="M2qAW+U6hDKcwcOWYiT+b9VHOy6irX93erXkEpP6UPGziP4Tt89tbslkmG90DAQ/RAQXiyxyY4VI391swfT4sQ==" saltValue="qMgqI4U5/0thO9gXTFLcNw==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0"/>
   <protectedRanges>
@@ -6548,6 +6548,33 @@
     <protectedRange sqref="H31:J31" name="Rango8_1"/>
   </protectedRanges>
   <mergeCells count="39">
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="A54:J54"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="B20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="F21:H21"/>
+    <mergeCell ref="H36:J36"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="I16:I18"/>
+    <mergeCell ref="J16:J18"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="F17:G17"/>
     <mergeCell ref="A14:J14"/>
     <mergeCell ref="A7:J7"/>
     <mergeCell ref="A8:J8"/>
@@ -6560,33 +6587,6 @@
     <mergeCell ref="F11:G11"/>
     <mergeCell ref="H11:I11"/>
     <mergeCell ref="A13:J13"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="I16:I18"/>
-    <mergeCell ref="J16:J18"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="B20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="F21:H21"/>
-    <mergeCell ref="H36:J36"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="A54:J54"/>
-    <mergeCell ref="A42:C42"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="A43:C43"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="D44:E44"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0.39370078740157483" top="0" bottom="0" header="0" footer="0"/>
@@ -6601,24 +6601,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
   <dimension ref="A1:Q51"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.33203125" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.33203125" style="296" customWidth="1"/>
-    <col min="2" max="2" width="2.109375" style="296" customWidth="1"/>
-    <col min="3" max="3" width="4.5546875" style="296" customWidth="1"/>
-    <col min="4" max="4" width="1.6640625" style="296" customWidth="1"/>
-    <col min="5" max="5" width="13.88671875" style="296" customWidth="1"/>
-    <col min="6" max="6" width="10.44140625" style="296" customWidth="1"/>
-    <col min="7" max="7" width="8.109375" style="296" customWidth="1"/>
-    <col min="8" max="8" width="6.5546875" style="296" customWidth="1"/>
-    <col min="9" max="11" width="10.5546875" style="296" customWidth="1"/>
-    <col min="12" max="12" width="1.5546875" style="296" customWidth="1"/>
-    <col min="13" max="13" width="13.5546875" style="296" customWidth="1"/>
-    <col min="14" max="14" width="6.44140625" style="296" customWidth="1"/>
-    <col min="15" max="15" width="8.5546875" style="296" customWidth="1"/>
+    <col min="1" max="1" width="11.28515625" style="296" customWidth="1"/>
+    <col min="2" max="2" width="2.140625" style="296" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="296" customWidth="1"/>
+    <col min="4" max="4" width="1.7109375" style="296" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" style="296" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" style="296" customWidth="1"/>
+    <col min="7" max="7" width="8.140625" style="296" customWidth="1"/>
+    <col min="8" max="8" width="6.5703125" style="296" customWidth="1"/>
+    <col min="9" max="11" width="10.5703125" style="296" customWidth="1"/>
+    <col min="12" max="12" width="1.5703125" style="296" customWidth="1"/>
+    <col min="13" max="13" width="13.5703125" style="296" customWidth="1"/>
+    <col min="14" max="14" width="6.42578125" style="296" customWidth="1"/>
+    <col min="15" max="15" width="8.5703125" style="296" customWidth="1"/>
     <col min="16" max="16" width="8" style="296" customWidth="1"/>
-    <col min="17" max="17" width="13.33203125" style="296" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="10.33203125" style="296"/>
+    <col min="17" max="17" width="13.28515625" style="296" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="10.28515625" style="296"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -6637,38 +6637,38 @@
       <c r="M1" s="295"/>
     </row>
     <row r="2" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="464" t="s">
+      <c r="A2" s="443" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="464"/>
-      <c r="C2" s="464"/>
-      <c r="D2" s="464"/>
-      <c r="E2" s="464"/>
-      <c r="F2" s="464"/>
-      <c r="G2" s="464"/>
-      <c r="H2" s="464"/>
-      <c r="I2" s="464"/>
-      <c r="J2" s="464"/>
-      <c r="K2" s="464"/>
-      <c r="L2" s="464"/>
-      <c r="M2" s="464"/>
+      <c r="B2" s="443"/>
+      <c r="C2" s="443"/>
+      <c r="D2" s="443"/>
+      <c r="E2" s="443"/>
+      <c r="F2" s="443"/>
+      <c r="G2" s="443"/>
+      <c r="H2" s="443"/>
+      <c r="I2" s="443"/>
+      <c r="J2" s="443"/>
+      <c r="K2" s="443"/>
+      <c r="L2" s="443"/>
+      <c r="M2" s="443"/>
     </row>
     <row r="3" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="465">
+      <c r="A3" s="444">
         <v>0</v>
       </c>
-      <c r="B3" s="465"/>
-      <c r="C3" s="465"/>
-      <c r="D3" s="465"/>
-      <c r="E3" s="465"/>
-      <c r="F3" s="465"/>
-      <c r="G3" s="465"/>
-      <c r="H3" s="465"/>
-      <c r="I3" s="465"/>
-      <c r="J3" s="465"/>
-      <c r="K3" s="465"/>
-      <c r="L3" s="465"/>
-      <c r="M3" s="465"/>
+      <c r="B3" s="444"/>
+      <c r="C3" s="444"/>
+      <c r="D3" s="444"/>
+      <c r="E3" s="444"/>
+      <c r="F3" s="444"/>
+      <c r="G3" s="444"/>
+      <c r="H3" s="444"/>
+      <c r="I3" s="444"/>
+      <c r="J3" s="444"/>
+      <c r="K3" s="444"/>
+      <c r="L3" s="444"/>
+      <c r="M3" s="444"/>
     </row>
     <row r="4" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6678,17 +6678,17 @@
       <c r="B5" s="298" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="476">
+      <c r="C5" s="455">
         <f>+FORMATO!N2</f>
         <v>0</v>
       </c>
-      <c r="D5" s="476"/>
-      <c r="E5" s="476"/>
-      <c r="F5" s="476"/>
-      <c r="G5" s="476"/>
-      <c r="H5" s="476"/>
-      <c r="I5" s="476"/>
-      <c r="J5" s="476"/>
+      <c r="D5" s="455"/>
+      <c r="E5" s="455"/>
+      <c r="F5" s="455"/>
+      <c r="G5" s="455"/>
+      <c r="H5" s="455"/>
+      <c r="I5" s="455"/>
+      <c r="J5" s="455"/>
       <c r="K5" s="299" t="s">
         <v>20</v>
       </c>
@@ -6706,17 +6706,17 @@
       <c r="B6" s="298" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="476">
+      <c r="C6" s="455">
         <f>+FORMATO!N3</f>
         <v>0</v>
       </c>
-      <c r="D6" s="476"/>
-      <c r="E6" s="476"/>
-      <c r="F6" s="476"/>
-      <c r="G6" s="476"/>
-      <c r="H6" s="476"/>
-      <c r="I6" s="476"/>
-      <c r="J6" s="476"/>
+      <c r="D6" s="455"/>
+      <c r="E6" s="455"/>
+      <c r="F6" s="455"/>
+      <c r="G6" s="455"/>
+      <c r="H6" s="455"/>
+      <c r="I6" s="455"/>
+      <c r="J6" s="455"/>
       <c r="K6" s="279" t="s">
         <v>119</v>
       </c>
@@ -6731,24 +6731,24 @@
       <c r="O6" s="303"/>
       <c r="P6" s="303"/>
     </row>
-    <row r="7" spans="1:16" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="297" t="s">
         <v>22</v>
       </c>
       <c r="B7" s="298" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="476">
+      <c r="C7" s="455">
         <f>+FORMATO!N4</f>
         <v>0</v>
       </c>
-      <c r="D7" s="476"/>
-      <c r="E7" s="476"/>
-      <c r="F7" s="476"/>
-      <c r="G7" s="476"/>
-      <c r="H7" s="476"/>
-      <c r="I7" s="476"/>
-      <c r="J7" s="476"/>
+      <c r="D7" s="455"/>
+      <c r="E7" s="455"/>
+      <c r="F7" s="455"/>
+      <c r="G7" s="455"/>
+      <c r="H7" s="455"/>
+      <c r="I7" s="455"/>
+      <c r="J7" s="455"/>
       <c r="K7" s="279" t="s">
         <v>158</v>
       </c>
@@ -6763,24 +6763,24 @@
       <c r="O7" s="303"/>
       <c r="P7" s="303"/>
     </row>
-    <row r="8" spans="1:16" ht="19.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="297" t="s">
         <v>23</v>
       </c>
       <c r="B8" s="298" t="s">
         <v>0</v>
       </c>
-      <c r="C8" s="476">
+      <c r="C8" s="455">
         <f>+FORMATO!N5</f>
         <v>0</v>
       </c>
-      <c r="D8" s="476"/>
-      <c r="E8" s="476"/>
-      <c r="F8" s="476"/>
-      <c r="G8" s="476"/>
-      <c r="H8" s="476"/>
-      <c r="I8" s="476"/>
-      <c r="J8" s="476"/>
+      <c r="D8" s="455"/>
+      <c r="E8" s="455"/>
+      <c r="F8" s="455"/>
+      <c r="G8" s="455"/>
+      <c r="H8" s="455"/>
+      <c r="I8" s="455"/>
+      <c r="J8" s="455"/>
       <c r="K8" s="304" t="s">
         <v>36</v>
       </c>
@@ -6788,7 +6788,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="305">
-        <f>+FORMATO!N8</f>
+        <f>+FORMATO!N9</f>
         <v>0</v>
       </c>
       <c r="N8" s="303"/>
@@ -6816,41 +6816,41 @@
       <c r="P9" s="303"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="468" t="s">
+      <c r="A10" s="447" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="469"/>
-      <c r="C10" s="469"/>
-      <c r="D10" s="469"/>
-      <c r="E10" s="469"/>
-      <c r="F10" s="469"/>
-      <c r="G10" s="469"/>
-      <c r="H10" s="469"/>
-      <c r="I10" s="469"/>
-      <c r="J10" s="469"/>
-      <c r="K10" s="469"/>
-      <c r="L10" s="469"/>
-      <c r="M10" s="470"/>
+      <c r="B10" s="448"/>
+      <c r="C10" s="448"/>
+      <c r="D10" s="448"/>
+      <c r="E10" s="448"/>
+      <c r="F10" s="448"/>
+      <c r="G10" s="448"/>
+      <c r="H10" s="448"/>
+      <c r="I10" s="448"/>
+      <c r="J10" s="448"/>
+      <c r="K10" s="448"/>
+      <c r="L10" s="448"/>
+      <c r="M10" s="449"/>
       <c r="N10" s="303"/>
       <c r="O10" s="303"/>
       <c r="P10" s="303"/>
     </row>
     <row r="11" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="471" t="s">
+      <c r="A11" s="450" t="s">
         <v>117</v>
       </c>
-      <c r="B11" s="472"/>
-      <c r="C11" s="472"/>
-      <c r="D11" s="472"/>
-      <c r="E11" s="472"/>
-      <c r="F11" s="472"/>
-      <c r="G11" s="472"/>
-      <c r="H11" s="472"/>
-      <c r="I11" s="472"/>
-      <c r="J11" s="472"/>
-      <c r="K11" s="472"/>
-      <c r="L11" s="472"/>
-      <c r="M11" s="473"/>
+      <c r="B11" s="451"/>
+      <c r="C11" s="451"/>
+      <c r="D11" s="451"/>
+      <c r="E11" s="451"/>
+      <c r="F11" s="451"/>
+      <c r="G11" s="451"/>
+      <c r="H11" s="451"/>
+      <c r="I11" s="451"/>
+      <c r="J11" s="451"/>
+      <c r="K11" s="451"/>
+      <c r="L11" s="451"/>
+      <c r="M11" s="452"/>
       <c r="N11" s="303"/>
       <c r="O11" s="303"/>
       <c r="P11" s="303"/>
@@ -6874,13 +6874,13 @@
       <c r="P12" s="303"/>
     </row>
     <row r="13" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="474" t="s">
+      <c r="A13" s="453" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="475"/>
-      <c r="C13" s="475"/>
-      <c r="D13" s="475"/>
-      <c r="E13" s="475"/>
+      <c r="B13" s="454"/>
+      <c r="C13" s="454"/>
+      <c r="D13" s="454"/>
+      <c r="E13" s="454"/>
       <c r="F13" s="318"/>
       <c r="G13" s="318"/>
       <c r="H13" s="318"/>
@@ -7011,15 +7011,15 @@
       <c r="A18" s="341"/>
       <c r="B18" s="342"/>
       <c r="C18" s="342"/>
-      <c r="D18" s="466"/>
-      <c r="E18" s="466"/>
+      <c r="D18" s="445"/>
+      <c r="E18" s="445"/>
       <c r="F18" s="342"/>
       <c r="G18" s="342"/>
       <c r="H18" s="342"/>
       <c r="I18" s="343"/>
       <c r="J18" s="343"/>
-      <c r="K18" s="467"/>
-      <c r="L18" s="467"/>
+      <c r="K18" s="446"/>
+      <c r="L18" s="446"/>
       <c r="M18" s="344"/>
       <c r="N18" s="303"/>
       <c r="O18" s="345"/>
@@ -7029,18 +7029,18 @@
       <c r="A19" s="346"/>
       <c r="B19" s="347"/>
       <c r="C19" s="347"/>
-      <c r="D19" s="443" t="s">
+      <c r="D19" s="456" t="s">
         <v>73</v>
       </c>
-      <c r="E19" s="444"/>
-      <c r="F19" s="444"/>
-      <c r="G19" s="444"/>
-      <c r="H19" s="445"/>
-      <c r="I19" s="461" t="s">
+      <c r="E19" s="457"/>
+      <c r="F19" s="457"/>
+      <c r="G19" s="457"/>
+      <c r="H19" s="458"/>
+      <c r="I19" s="474" t="s">
         <v>72</v>
       </c>
-      <c r="J19" s="461"/>
-      <c r="K19" s="462"/>
+      <c r="J19" s="474"/>
+      <c r="K19" s="475"/>
       <c r="L19" s="348"/>
       <c r="M19" s="349"/>
       <c r="N19" s="303"/>
@@ -7051,11 +7051,11 @@
       <c r="A20" s="350"/>
       <c r="B20" s="295"/>
       <c r="C20" s="295"/>
-      <c r="D20" s="446"/>
-      <c r="E20" s="447"/>
-      <c r="F20" s="447"/>
-      <c r="G20" s="447"/>
-      <c r="H20" s="448"/>
+      <c r="D20" s="459"/>
+      <c r="E20" s="460"/>
+      <c r="F20" s="460"/>
+      <c r="G20" s="460"/>
+      <c r="H20" s="461"/>
       <c r="I20" s="351">
         <v>1</v>
       </c>
@@ -7127,8 +7127,8 @@
         <f>+Datos!I14</f>
         <v>0</v>
       </c>
-      <c r="L22" s="455"/>
-      <c r="M22" s="454"/>
+      <c r="L22" s="468"/>
+      <c r="M22" s="467"/>
       <c r="N22" s="303"/>
       <c r="O22" s="364"/>
       <c r="P22" s="303"/>
@@ -7158,8 +7158,8 @@
         <f>+Datos!I15</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="L23" s="453"/>
-      <c r="M23" s="454"/>
+      <c r="L23" s="466"/>
+      <c r="M23" s="467"/>
       <c r="N23" s="303"/>
       <c r="O23" s="303"/>
       <c r="P23" s="364"/>
@@ -7177,12 +7177,12 @@
       <c r="H24" s="360" t="s">
         <v>1</v>
       </c>
-      <c r="I24" s="456" t="e">
+      <c r="I24" s="469" t="e">
         <f>+Datos!G16</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="J24" s="457"/>
-      <c r="K24" s="458"/>
+      <c r="J24" s="470"/>
+      <c r="K24" s="471"/>
       <c r="L24" s="369"/>
       <c r="M24" s="362"/>
       <c r="N24" s="303"/>
@@ -7244,10 +7244,10 @@
       <c r="C28" s="386"/>
       <c r="D28" s="367"/>
       <c r="E28" s="369"/>
-      <c r="F28" s="459" t="s">
+      <c r="F28" s="472" t="s">
         <v>176</v>
       </c>
-      <c r="G28" s="460"/>
+      <c r="G28" s="473"/>
       <c r="M28" s="384"/>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.25">
@@ -7270,11 +7270,11 @@
       <c r="C30" s="386"/>
       <c r="D30" s="367"/>
       <c r="E30" s="369"/>
-      <c r="F30" s="449">
+      <c r="F30" s="462">
         <f>+Datos!E25</f>
         <v>0</v>
       </c>
-      <c r="G30" s="450"/>
+      <c r="G30" s="463"/>
       <c r="M30" s="384"/>
     </row>
     <row r="31" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -7285,11 +7285,11 @@
       <c r="C31" s="386"/>
       <c r="D31" s="367"/>
       <c r="E31" s="369"/>
-      <c r="F31" s="449">
+      <c r="F31" s="462">
         <f>+Datos!E26</f>
         <v>0</v>
       </c>
-      <c r="G31" s="450"/>
+      <c r="G31" s="463"/>
       <c r="M31" s="384"/>
     </row>
     <row r="32" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -7326,100 +7326,100 @@
       <c r="M34" s="393"/>
     </row>
     <row r="35" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="463" t="s">
+      <c r="A35" s="476" t="s">
         <v>171</v>
       </c>
-      <c r="B35" s="463"/>
-      <c r="C35" s="463"/>
-      <c r="D35" s="463"/>
-      <c r="E35" s="463"/>
-      <c r="F35" s="463"/>
-      <c r="G35" s="463"/>
-      <c r="H35" s="463"/>
-      <c r="I35" s="463"/>
-      <c r="J35" s="463"/>
-      <c r="K35" s="463"/>
-      <c r="L35" s="463"/>
-      <c r="M35" s="463"/>
-    </row>
-    <row r="36" spans="1:16" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="452" t="s">
+      <c r="B35" s="476"/>
+      <c r="C35" s="476"/>
+      <c r="D35" s="476"/>
+      <c r="E35" s="476"/>
+      <c r="F35" s="476"/>
+      <c r="G35" s="476"/>
+      <c r="H35" s="476"/>
+      <c r="I35" s="476"/>
+      <c r="J35" s="476"/>
+      <c r="K35" s="476"/>
+      <c r="L35" s="476"/>
+      <c r="M35" s="476"/>
+    </row>
+    <row r="36" spans="1:16" ht="34.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="465" t="s">
         <v>172</v>
       </c>
-      <c r="B36" s="452"/>
-      <c r="C36" s="452"/>
-      <c r="D36" s="452"/>
-      <c r="E36" s="452"/>
-      <c r="F36" s="452"/>
-      <c r="G36" s="452"/>
-      <c r="H36" s="452"/>
-      <c r="I36" s="452"/>
-      <c r="J36" s="452"/>
-      <c r="K36" s="452"/>
-      <c r="L36" s="452"/>
-      <c r="M36" s="452"/>
-    </row>
-    <row r="37" spans="1:16" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="452" t="s">
+      <c r="B36" s="465"/>
+      <c r="C36" s="465"/>
+      <c r="D36" s="465"/>
+      <c r="E36" s="465"/>
+      <c r="F36" s="465"/>
+      <c r="G36" s="465"/>
+      <c r="H36" s="465"/>
+      <c r="I36" s="465"/>
+      <c r="J36" s="465"/>
+      <c r="K36" s="465"/>
+      <c r="L36" s="465"/>
+      <c r="M36" s="465"/>
+    </row>
+    <row r="37" spans="1:16" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="465" t="s">
         <v>173</v>
       </c>
-      <c r="B37" s="452"/>
-      <c r="C37" s="452"/>
-      <c r="D37" s="452"/>
-      <c r="E37" s="452"/>
-      <c r="F37" s="452"/>
-      <c r="G37" s="452"/>
-      <c r="H37" s="452"/>
-      <c r="I37" s="452"/>
-      <c r="J37" s="452"/>
-      <c r="K37" s="452"/>
-      <c r="L37" s="452"/>
-      <c r="M37" s="452"/>
+      <c r="B37" s="465"/>
+      <c r="C37" s="465"/>
+      <c r="D37" s="465"/>
+      <c r="E37" s="465"/>
+      <c r="F37" s="465"/>
+      <c r="G37" s="465"/>
+      <c r="H37" s="465"/>
+      <c r="I37" s="465"/>
+      <c r="J37" s="465"/>
+      <c r="K37" s="465"/>
+      <c r="L37" s="465"/>
+      <c r="M37" s="465"/>
       <c r="N37" s="303"/>
       <c r="O37" s="303"/>
       <c r="P37" s="303"/>
     </row>
-    <row r="38" spans="1:16" ht="25.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="452" t="s">
+    <row r="38" spans="1:16" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="465" t="s">
         <v>174</v>
       </c>
-      <c r="B38" s="452"/>
-      <c r="C38" s="452"/>
-      <c r="D38" s="452"/>
-      <c r="E38" s="452"/>
-      <c r="F38" s="452"/>
-      <c r="G38" s="452"/>
-      <c r="H38" s="452"/>
-      <c r="I38" s="452"/>
-      <c r="J38" s="452"/>
-      <c r="K38" s="452"/>
-      <c r="L38" s="452"/>
-      <c r="M38" s="452"/>
+      <c r="B38" s="465"/>
+      <c r="C38" s="465"/>
+      <c r="D38" s="465"/>
+      <c r="E38" s="465"/>
+      <c r="F38" s="465"/>
+      <c r="G38" s="465"/>
+      <c r="H38" s="465"/>
+      <c r="I38" s="465"/>
+      <c r="J38" s="465"/>
+      <c r="K38" s="465"/>
+      <c r="L38" s="465"/>
+      <c r="M38" s="465"/>
       <c r="N38" s="303"/>
       <c r="O38" s="303"/>
       <c r="P38" s="303"/>
     </row>
     <row r="39" spans="1:16" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="451" t="s">
+      <c r="A39" s="464" t="s">
         <v>175</v>
       </c>
-      <c r="B39" s="451"/>
-      <c r="C39" s="451"/>
-      <c r="D39" s="451"/>
-      <c r="E39" s="451"/>
-      <c r="F39" s="451"/>
-      <c r="G39" s="451"/>
-      <c r="H39" s="451"/>
-      <c r="I39" s="451"/>
-      <c r="J39" s="451"/>
-      <c r="K39" s="451"/>
-      <c r="L39" s="451"/>
-      <c r="M39" s="451"/>
+      <c r="B39" s="464"/>
+      <c r="C39" s="464"/>
+      <c r="D39" s="464"/>
+      <c r="E39" s="464"/>
+      <c r="F39" s="464"/>
+      <c r="G39" s="464"/>
+      <c r="H39" s="464"/>
+      <c r="I39" s="464"/>
+      <c r="J39" s="464"/>
+      <c r="K39" s="464"/>
+      <c r="L39" s="464"/>
+      <c r="M39" s="464"/>
       <c r="N39" s="303"/>
       <c r="O39" s="303"/>
       <c r="P39" s="303"/>
     </row>
-    <row r="40" spans="1:16" ht="4.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:16" ht="4.9000000000000004" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="394"/>
       <c r="B40" s="394"/>
       <c r="C40" s="394"/>
@@ -7451,7 +7451,7 @@
       <c r="O41" s="303"/>
       <c r="P41" s="303"/>
     </row>
-    <row r="42" spans="1:16" ht="25.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:16" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="325"/>
       <c r="B42" s="325"/>
       <c r="C42" s="325"/>
@@ -7595,7 +7595,7 @@
       <c r="L49" s="295"/>
       <c r="M49" s="295"/>
     </row>
-    <row r="50" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="295"/>
       <c r="B50" s="295"/>
       <c r="C50" s="295"/>
@@ -7610,7 +7610,7 @@
       <c r="L50" s="295"/>
       <c r="M50" s="295"/>
     </row>
-    <row r="51" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="51" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="8NM1+p6p3LesDUstMxFGHu0zYxm1d4zXGYtLxhJOWwI+xJ9//NVS0q83GcKW2Ki+XgVMpMuspxvNsKuxOQLOxg==" saltValue="QYjBUm0XnOsAQh3sj8wCVA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <protectedRanges>
@@ -7619,17 +7619,6 @@
     <protectedRange sqref="C5:E6" name="Rango3_3_1_1_1_1_1_2_1_1"/>
   </protectedRanges>
   <mergeCells count="24">
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="A10:M10"/>
-    <mergeCell ref="A11:M11"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="C5:J5"/>
-    <mergeCell ref="C6:J6"/>
-    <mergeCell ref="C7:J7"/>
-    <mergeCell ref="C8:J8"/>
     <mergeCell ref="D19:H20"/>
     <mergeCell ref="F30:G30"/>
     <mergeCell ref="F31:G31"/>
@@ -7643,6 +7632,17 @@
     <mergeCell ref="A35:M35"/>
     <mergeCell ref="A36:M36"/>
     <mergeCell ref="A38:M38"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="A10:M10"/>
+    <mergeCell ref="A11:M11"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="C5:J5"/>
+    <mergeCell ref="C6:J6"/>
+    <mergeCell ref="C7:J7"/>
+    <mergeCell ref="C8:J8"/>
   </mergeCells>
   <dataValidations disablePrompts="1" count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F28:G28" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -7666,14 +7666,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:O34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.33203125" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.44140625" style="28" customWidth="1"/>
-    <col min="2" max="9" width="11.6640625" style="28" customWidth="1"/>
-    <col min="10" max="10" width="1.5546875" style="28" customWidth="1"/>
-    <col min="11" max="11" width="13.5546875" style="28" customWidth="1"/>
-    <col min="12" max="16" width="16.88671875" style="28" customWidth="1"/>
-    <col min="17" max="16384" width="10.33203125" style="28"/>
+    <col min="1" max="1" width="6.42578125" style="28" customWidth="1"/>
+    <col min="2" max="9" width="11.7109375" style="28" customWidth="1"/>
+    <col min="10" max="10" width="1.5703125" style="28" customWidth="1"/>
+    <col min="11" max="11" width="13.5703125" style="28" customWidth="1"/>
+    <col min="12" max="16" width="16.85546875" style="28" customWidth="1"/>
+    <col min="17" max="16384" width="10.28515625" style="28"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8394,7 +8394,7 @@
       <c r="J32" s="41"/>
       <c r="K32" s="41"/>
     </row>
-    <row r="33" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="41"/>
       <c r="B33" s="58"/>
       <c r="C33" s="58"/>
@@ -8407,7 +8407,7 @@
       <c r="J33" s="41"/>
       <c r="K33" s="41"/>
     </row>
-    <row r="34" spans="1:11" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" spans="1:11" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="30HaiR52nqiYotLJpI1mB2lORNPbDurlcC6410k5mvSvnGiAmVghg7imMzZoWOpv930Refz4w5FF+iObjCt0iQ==" saltValue="+OutNn2WwZIf1rmOnZwRlA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <protectedRanges>
@@ -8444,22 +8444,22 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:X58"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.44140625" style="15" customWidth="1"/>
-    <col min="2" max="5" width="10.44140625" style="15" customWidth="1"/>
-    <col min="6" max="8" width="13.109375" style="15" customWidth="1"/>
-    <col min="9" max="9" width="18.109375" style="15" customWidth="1"/>
-    <col min="10" max="10" width="15.44140625" style="15" customWidth="1"/>
+    <col min="1" max="1" width="19.42578125" style="15" customWidth="1"/>
+    <col min="2" max="5" width="10.42578125" style="15" customWidth="1"/>
+    <col min="6" max="8" width="13.140625" style="15" customWidth="1"/>
+    <col min="9" max="9" width="18.140625" style="15" customWidth="1"/>
+    <col min="10" max="10" width="15.42578125" style="15" customWidth="1"/>
     <col min="11" max="12" width="12" style="15" customWidth="1"/>
-    <col min="13" max="16" width="12.6640625" style="15" customWidth="1"/>
-    <col min="17" max="17" width="14.6640625" style="15" customWidth="1"/>
-    <col min="18" max="20" width="12.109375" style="15" customWidth="1"/>
+    <col min="13" max="16" width="12.7109375" style="15" customWidth="1"/>
+    <col min="17" max="17" width="14.7109375" style="15" customWidth="1"/>
+    <col min="18" max="20" width="12.140625" style="15" customWidth="1"/>
     <col min="21" max="24" width="13" style="15" customWidth="1"/>
-    <col min="25" max="16384" width="11.44140625" style="15"/>
+    <col min="25" max="16384" width="11.42578125" style="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="516"/>
       <c r="B1" s="516"/>
       <c r="C1" s="507" t="s">
@@ -8477,7 +8477,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="516"/>
       <c r="B2" s="516"/>
       <c r="C2" s="510"/>
@@ -8493,7 +8493,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="516"/>
       <c r="B3" s="516"/>
       <c r="C3" s="510"/>
@@ -8509,7 +8509,7 @@
         <v>46146</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="516"/>
       <c r="B4" s="516"/>
       <c r="C4" s="513"/>
@@ -8525,7 +8525,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="170" t="s">
         <v>50</v>
       </c>
@@ -8541,7 +8541,7 @@
       <c r="I6" s="17"/>
       <c r="J6" s="16"/>
     </row>
-    <row r="7" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="170" t="s">
         <v>49</v>
       </c>
@@ -8557,7 +8557,7 @@
       <c r="I7" s="17"/>
       <c r="J7" s="16"/>
     </row>
-    <row r="8" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="170" t="s">
         <v>48</v>
       </c>
@@ -8573,7 +8573,7 @@
       <c r="I8" s="17"/>
       <c r="J8" s="16"/>
     </row>
-    <row r="9" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="171" t="s">
         <v>161</v>
       </c>
@@ -8589,7 +8589,7 @@
       <c r="I9" s="17"/>
       <c r="J9" s="16"/>
     </row>
-    <row r="11" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="172" t="s">
         <v>168</v>
       </c>
@@ -8602,7 +8602,7 @@
       <c r="H11" s="167"/>
       <c r="I11" s="167"/>
     </row>
-    <row r="12" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="167"/>
       <c r="B12" s="167"/>
       <c r="C12" s="167"/>
@@ -8613,7 +8613,7 @@
       <c r="H12" s="167"/>
       <c r="I12" s="167"/>
     </row>
-    <row r="13" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="173" t="s">
         <v>104</v>
       </c>
@@ -8628,7 +8628,7 @@
       <c r="H13" s="167"/>
       <c r="I13" s="167"/>
     </row>
-    <row r="14" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="167"/>
       <c r="B14" s="167"/>
       <c r="C14" s="167"/>
@@ -8639,7 +8639,7 @@
       <c r="H14" s="167"/>
       <c r="I14" s="167"/>
     </row>
-    <row r="15" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="176" t="s">
         <v>108</v>
       </c>
@@ -8652,7 +8652,7 @@
       <c r="H15" s="167"/>
       <c r="I15" s="167"/>
     </row>
-    <row r="16" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="176" t="s">
         <v>109</v>
       </c>
@@ -8665,7 +8665,7 @@
       <c r="H16" s="167"/>
       <c r="I16" s="167"/>
     </row>
-    <row r="17" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="176" t="s">
         <v>110</v>
       </c>
@@ -8678,7 +8678,7 @@
       <c r="H17" s="167"/>
       <c r="I17" s="167"/>
     </row>
-    <row r="18" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="167"/>
       <c r="B18" s="167"/>
       <c r="C18" s="167"/>
@@ -8689,7 +8689,7 @@
       <c r="H18" s="167"/>
       <c r="I18" s="167"/>
     </row>
-    <row r="19" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="173" t="s">
         <v>106</v>
       </c>
@@ -8702,7 +8702,7 @@
       <c r="H19" s="167"/>
       <c r="I19" s="167"/>
     </row>
-    <row r="20" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="167"/>
       <c r="B20" s="167"/>
       <c r="C20" s="167"/>
@@ -8713,7 +8713,7 @@
       <c r="H20" s="167"/>
       <c r="I20" s="167"/>
     </row>
-    <row r="21" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="176" t="s">
         <v>111</v>
       </c>
@@ -8726,7 +8726,7 @@
       <c r="H21" s="167"/>
       <c r="I21" s="167"/>
     </row>
-    <row r="22" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="167"/>
       <c r="B22" s="167"/>
       <c r="C22" s="167"/>
@@ -8737,7 +8737,7 @@
       <c r="H22" s="167"/>
       <c r="I22" s="167"/>
     </row>
-    <row r="23" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="172" t="s">
         <v>107</v>
       </c>
@@ -8750,7 +8750,7 @@
       <c r="H23" s="167"/>
       <c r="I23" s="167"/>
     </row>
-    <row r="24" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="167"/>
       <c r="B24" s="167"/>
       <c r="C24" s="167"/>
@@ -8761,11 +8761,11 @@
       <c r="H24" s="167"/>
       <c r="I24" s="167"/>
     </row>
-    <row r="25" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:24" ht="54.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="26" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="27" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="28" spans="1:24" ht="54.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="29" spans="1:24" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F29" s="91"/>
       <c r="H29" s="91"/>
       <c r="I29" s="91"/>
@@ -8780,7 +8780,7 @@
       <c r="T29" s="167"/>
       <c r="U29" s="167"/>
     </row>
-    <row r="30" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:24" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="L30" s="166"/>
       <c r="M30" s="167"/>
       <c r="N30" s="167"/>
@@ -8792,7 +8792,7 @@
       <c r="T30" s="167"/>
       <c r="U30" s="167"/>
     </row>
-    <row r="31" spans="1:24" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:24" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="L31" s="168"/>
       <c r="M31" s="168"/>
       <c r="N31" s="168"/>
@@ -8804,7 +8804,7 @@
       <c r="T31" s="168"/>
       <c r="U31" s="168"/>
     </row>
-    <row r="32" spans="1:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:24" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A32" s="139" t="s">
         <v>47</v>
       </c>
@@ -8878,7 +8878,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="33" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="126" t="s">
         <v>59</v>
       </c>
@@ -8919,7 +8919,7 @@
       <c r="W33" s="112"/>
       <c r="X33" s="128"/>
     </row>
-    <row r="34" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="122" t="s">
         <v>64</v>
       </c>
@@ -8999,7 +8999,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="35" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="124" t="s">
         <v>60</v>
       </c>
@@ -9073,7 +9073,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="36" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="122" t="s">
         <v>65</v>
       </c>
@@ -9153,7 +9153,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="37" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:24" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="124" t="s">
         <v>60</v>
       </c>
@@ -9370,7 +9370,7 @@
       <c r="W40" s="137"/>
       <c r="X40" s="137"/>
     </row>
-    <row r="41" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="111"/>
       <c r="D41" s="111"/>
       <c r="E41" s="111"/>
@@ -9380,7 +9380,7 @@
       <c r="I41" s="111"/>
       <c r="J41" s="111"/>
     </row>
-    <row r="42" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="111"/>
       <c r="B42" s="14"/>
       <c r="C42" s="13"/>
@@ -9392,7 +9392,7 @@
       <c r="I42" s="111"/>
       <c r="J42" s="111"/>
     </row>
-    <row r="43" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="148"/>
       <c r="B43" s="152" t="str">
         <f>A34</f>
@@ -9413,7 +9413,7 @@
       <c r="I43" s="111"/>
       <c r="J43" s="111"/>
     </row>
-    <row r="44" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="148"/>
       <c r="B44" s="152" t="str">
         <f>A36</f>
@@ -9434,7 +9434,7 @@
       <c r="I44" s="111"/>
       <c r="J44" s="111"/>
     </row>
-    <row r="45" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B45" s="152" t="str">
         <f>A38</f>
         <v>factor de presición</v>
@@ -9454,7 +9454,7 @@
       <c r="I45" s="111"/>
       <c r="J45" s="111"/>
     </row>
-    <row r="46" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="505"/>
       <c r="B46" s="506"/>
       <c r="C46" s="151" t="e">
@@ -9469,7 +9469,7 @@
       <c r="I46" s="111"/>
       <c r="J46" s="111"/>
     </row>
-    <row r="47" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A47" s="111"/>
       <c r="B47" s="111"/>
       <c r="C47" s="111"/>
@@ -9481,7 +9481,7 @@
       <c r="I47" s="111"/>
       <c r="J47" s="111"/>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" s="290" t="s">
         <v>162</v>
       </c>
@@ -9499,7 +9499,7 @@
       </c>
       <c r="H55" s="521"/>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56" s="167"/>
       <c r="B56" s="167"/>
       <c r="C56" s="167"/>
@@ -9509,7 +9509,7 @@
       <c r="G56" s="167"/>
       <c r="H56" s="167"/>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57" s="287" t="s">
         <v>166</v>
       </c>
@@ -9527,7 +9527,7 @@
       </c>
       <c r="H57" s="503"/>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="167"/>
       <c r="B58" s="167"/>
       <c r="C58" s="167"/>
@@ -9562,24 +9562,24 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A2:G30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" style="15"/>
-    <col min="2" max="2" width="13.5546875" style="15" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" style="15"/>
+    <col min="2" max="2" width="13.5703125" style="15" customWidth="1"/>
     <col min="3" max="3" width="12" style="15" customWidth="1"/>
-    <col min="4" max="6" width="11.44140625" style="15"/>
-    <col min="7" max="7" width="14.44140625" style="15" customWidth="1"/>
-    <col min="8" max="8" width="11.44140625" style="15"/>
-    <col min="9" max="9" width="11.88671875" style="15" customWidth="1"/>
-    <col min="10" max="16384" width="11.44140625" style="15"/>
+    <col min="4" max="6" width="11.42578125" style="15"/>
+    <col min="7" max="7" width="14.42578125" style="15" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" style="15"/>
+    <col min="9" max="9" width="11.85546875" style="15" customWidth="1"/>
+    <col min="10" max="16384" width="11.42578125" style="15"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="100" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B4" s="101" t="str">
         <f>+Datos!B13</f>
         <v>Lectura de la arcilla</v>
@@ -9597,7 +9597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B5" s="101" t="str">
         <f>+Datos!B14</f>
         <v>Lectura de la arena</v>
@@ -9615,7 +9615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="523" t="s">
         <v>58</v>
       </c>
@@ -9625,14 +9625,14 @@
       <c r="E9" s="26"/>
       <c r="F9" s="26"/>
     </row>
-    <row r="10" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="21"/>
       <c r="C10" s="21"/>
       <c r="D10" s="21"/>
       <c r="E10" s="27"/>
       <c r="F10" s="94"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="102" t="s">
         <v>98</v>
       </c>
@@ -9640,13 +9640,13 @@
       <c r="F11" s="94"/>
       <c r="G11" s="94"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="103"/>
       <c r="B12" s="91"/>
       <c r="F12" s="94"/>
       <c r="G12" s="94"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="104">
         <v>1</v>
       </c>
@@ -9657,7 +9657,7 @@
         <v>381.6</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="104">
         <v>2</v>
       </c>
@@ -9671,7 +9671,7 @@
       <c r="F14" s="95"/>
       <c r="G14" s="95"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="104">
         <v>3</v>
       </c>
@@ -9685,7 +9685,7 @@
       <c r="F15" s="95"/>
       <c r="G15" s="95"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="104">
         <v>4</v>
       </c>
@@ -9694,7 +9694,7 @@
       <c r="F16" s="95"/>
       <c r="G16" s="95"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="525" t="s">
         <v>96</v>
       </c>
@@ -9704,7 +9704,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="525"/>
       <c r="B18" s="525"/>
       <c r="C18" s="108">
@@ -9714,7 +9714,7 @@
       <c r="F18" s="95"/>
       <c r="G18" s="95"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="20"/>
       <c r="B19" s="21"/>
       <c r="C19" s="21"/>
@@ -9722,66 +9722,66 @@
       <c r="F19" s="95"/>
       <c r="G19" s="95"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B20" s="21"/>
       <c r="C20" s="21"/>
       <c r="D20" s="21"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="504"/>
       <c r="B21" s="21"/>
       <c r="C21" s="21"/>
       <c r="D21" s="21"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" s="504"/>
       <c r="B22" s="21"/>
       <c r="C22" s="21"/>
       <c r="D22" s="21"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="504"/>
       <c r="B23" s="21"/>
       <c r="C23" s="21"/>
       <c r="D23" s="21"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="504"/>
       <c r="B24" s="21"/>
       <c r="C24" s="21"/>
       <c r="D24" s="21"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" s="522"/>
       <c r="B25" s="21"/>
       <c r="C25" s="21"/>
       <c r="D25" s="21"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="522"/>
       <c r="B26" s="21"/>
       <c r="C26" s="21"/>
       <c r="D26" s="21"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" s="522"/>
       <c r="B27" s="21"/>
       <c r="C27" s="21"/>
       <c r="D27" s="21"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" s="522"/>
       <c r="B28" s="21"/>
       <c r="C28" s="21"/>
       <c r="D28" s="21"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" s="20"/>
       <c r="B29" s="22"/>
       <c r="C29" s="23"/>
       <c r="D29" s="22"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C30" s="24"/>
       <c r="D30" s="25"/>
     </row>
@@ -9801,30 +9801,30 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="39.6640625" style="186" customWidth="1"/>
-    <col min="2" max="16384" width="11.5546875" style="186"/>
+    <col min="1" max="1" width="39.7109375" style="186" customWidth="1"/>
+    <col min="2" max="16384" width="11.5703125" style="186"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="9.6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="9.6" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="187"/>
     </row>
-    <row r="3" spans="1:11" ht="6.6" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:11" ht="6.6" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="292" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="93"/>
       <c r="H5" s="188"/>
       <c r="I5" s="526"/>
       <c r="J5" s="526"/>
       <c r="K5" s="526"/>
     </row>
-    <row r="6" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="93" t="s">
         <v>94</v>
       </c>
@@ -9836,7 +9836,7 @@
       <c r="J6" s="191"/>
       <c r="K6" s="191"/>
     </row>
-    <row r="7" spans="1:11" ht="7.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="7.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="93"/>
       <c r="B7" s="192"/>
       <c r="H7" s="288"/>
@@ -9844,7 +9844,7 @@
       <c r="J7" s="191"/>
       <c r="K7" s="191"/>
     </row>
-    <row r="8" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="193" t="s">
         <v>120</v>
       </c>
@@ -9855,7 +9855,7 @@
       <c r="D8" s="527"/>
       <c r="E8" s="92"/>
     </row>
-    <row r="9" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="193" t="s">
         <v>121</v>
       </c>
@@ -9882,18 +9882,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr codeName="Hoja3"/>
   <dimension ref="A2:M9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="10.44140625" customWidth="1"/>
-    <col min="3" max="3" width="18.33203125" customWidth="1"/>
+    <col min="1" max="2" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="18.28515625" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="6" max="6" width="12.44140625" customWidth="1"/>
-    <col min="11" max="11" width="17.6640625" customWidth="1"/>
-    <col min="12" max="12" width="12.44140625" customWidth="1"/>
-    <col min="13" max="13" width="15.44140625" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="11" max="11" width="17.7109375" customWidth="1"/>
+    <col min="12" max="12" width="12.42578125" customWidth="1"/>
+    <col min="13" max="13" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="528" t="s">
         <v>11</v>
       </c>
@@ -9932,7 +9932,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="7">
         <v>4400</v>
       </c>
@@ -9978,7 +9978,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="6" t="str">
@@ -10015,7 +10015,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <f>+B3+1</f>
         <v>4402</v>
@@ -10058,7 +10058,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="6" t="str">
@@ -10095,7 +10095,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <f>+B5+1</f>
         <v>4404</v>
@@ -10138,7 +10138,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="6" t="str">
@@ -10175,7 +10175,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:B2"/>

</xml_diff>